<commit_message>
progress: 39 village workbooks (randomwalk-TRX50-WS 2026-10-09T16:10:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Edur_13.477828_80.078782.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Edur_13.477828_80.078782.xlsx
@@ -494,11 +494,6 @@
           <t>103</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>1, 10A, 10B, 2, 3, 4, 5, 6, 7, 8A, 8B, 9</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -506,11 +501,6 @@
           <t>104</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>1, 10A, 10B, 10C, 10D, 11, 12, 13, 2, 3, 4, 5, 6, 7, 8A, 8B, 9A, 9B, 9C</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -518,11 +508,6 @@
           <t>105</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>1, 10, 11A, 11B, 12, 2A, 2B, 2C, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -530,11 +515,6 @@
           <t>106</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>1, 10A, 10B, 11, 12, 13, 14, 2, 3, 4, 5, 6, 7, 8A, 8B, 9</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -542,11 +522,6 @@
           <t>107</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 1A, 1B, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -554,11 +529,6 @@
           <t>108</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -566,11 +536,6 @@
           <t>109</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -578,11 +543,6 @@
           <t>11</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 2, 3, 4, 5, 6A, 6B, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -590,11 +550,6 @@
           <t>110</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>1, 2, 3A, 3B, 4, 5</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -602,11 +557,6 @@
           <t>111</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5A, 5B, 6, 7, 8A, 8B</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -614,11 +564,6 @@
           <t>112</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 3A, 3B, 4, 5, 6A, 6B, 6C, 6D, 6E, 7, 8, 9A, 9B</t>
-        </is>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -626,11 +571,6 @@
           <t>113</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>10, 11, 12, 1A, 1B, 1C, 1D, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -638,11 +578,6 @@
           <t>114</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>10, 11A, 11B, 12A, 12B, 13, 1A, 1B, 2, 3, 4, 5, 6, 7, 8A, 8B, 9</t>
-        </is>
-      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -650,11 +585,6 @@
           <t>115</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>1, 2, 3A, 3B, 3C, 3D, 3E, 4, 5, 6</t>
-        </is>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -662,11 +592,6 @@
           <t>116</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>1, 10, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -674,11 +599,6 @@
           <t>117</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -686,11 +606,6 @@
           <t>118</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -698,11 +613,6 @@
           <t>119</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -710,11 +620,6 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -722,11 +627,6 @@
           <t>120</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -734,11 +634,6 @@
           <t>121</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>1A, 1B, 1C, 2, 3A, 3B, 4, 5, 6</t>
-        </is>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -746,11 +641,6 @@
           <t>122</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 1A, 1B, 2, 20, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -758,11 +648,6 @@
           <t>123</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 2A, 2B, 3, 4A, 4B, 5A, 5B, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -770,11 +655,6 @@
           <t>124</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>1A, 1B, 1C, 1D, 2A, 2B, 3A, 3B, 4, 5</t>
-        </is>
-      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -782,11 +662,6 @@
           <t>125</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>1A, 1B, 1C, 2, 3A, 3B, 3C, 4A, 4B, 5A, 5B, 6</t>
-        </is>
-      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -794,11 +669,6 @@
           <t>126</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 2C, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -806,11 +676,6 @@
           <t>127</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>10A, 10B, 11, 12, 13, 14A1, 14A2, 14B, 15A, 15B, 1A, 1B, 2A, 2B, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -818,11 +683,6 @@
           <t>128</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>10A, 10B, 11, 12A, 12B, 13, 14, 1A1, 1B, 1C, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -830,11 +690,6 @@
           <t>129</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>10, 11, 12, 13A, 13B, 13C, 13D, 14, 15, 16, 1A, 1B, 1C, 2, 3, 4, 5, 6A, 6B, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -842,11 +697,6 @@
           <t>13</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>10, 11, 12, 1A, 1B, 2, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -854,11 +704,6 @@
           <t>130</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -866,11 +711,6 @@
           <t>131</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -878,11 +718,6 @@
           <t>132</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>1, 10, 2, 3, 4, 5, 6A, 6B, 6C1, 6C2, 6D1, 6D2, 6E, 6F1, 6F2, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -890,11 +725,6 @@
           <t>133</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>1, 10A, 10B, 10C, 11, 12, 13, 14, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -902,11 +732,6 @@
           <t>134</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14A, 14B, 2, 3, 4, 5, 6, 7, 8, 9A, 9B</t>
-        </is>
-      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -914,11 +739,6 @@
           <t>135</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
-      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -926,11 +746,6 @@
           <t>136</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -938,11 +753,6 @@
           <t>137</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>1, 10, 11A, 11B, 12A, 12B, 2, 3, 4A, 4B, 5A, 5B, 5C, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -950,11 +760,6 @@
           <t>138</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>1A, 1B, 1C, 1D, 1E, 1F, 1G, 1H, 1I, 2A, 2B, 3, 4</t>
-        </is>
-      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -962,11 +767,6 @@
           <t>139</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>10, 11, 12, 1A, 1B, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -974,11 +774,6 @@
           <t>14</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -986,11 +781,6 @@
           <t>140</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -998,11 +788,6 @@
           <t>141</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>1, 10, 2, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1010,11 +795,6 @@
           <t>142</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>1, 10A, 10B, 11A, 11B, 11C, 11D, 2, 3, 4, 5, 6, 7, 8A, 8B, 9</t>
-        </is>
-      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1022,11 +802,6 @@
           <t>143</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1034,11 +809,6 @@
           <t>144</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>1, 10, 2, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1046,11 +816,6 @@
           <t>145</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13A1, 13A2, 13B, 14A, 14B, 14C, 15A, 15B, 16A, 16B, 16C, 16D, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1058,11 +823,6 @@
           <t>146</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>1, 10, 2, 3, 4A, 4B, 5A, 5B, 6, 7A, 7B, 8, 9A, 9B1, 9B2</t>
-        </is>
-      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1070,11 +830,6 @@
           <t>147</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>1, 10, 11A, 11B, 12, 13, 14, 2A, 2B, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1082,11 +837,6 @@
           <t>148</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>10A, 10B, 1A, 1B, 2A1, 2A2, 2B, 3, 4, 5, 6, 7A, 7B, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1094,11 +844,6 @@
           <t>149</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 19A, 19B, 1A, 1B, 1C, 1D, 2, 20, 21A, 21B, 22, 23A, 23B, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1106,11 +851,6 @@
           <t>15</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1118,11 +858,6 @@
           <t>150</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>1, 10, 11A, 11B, 12A, 12B, 13, 2, 3, 4, 5, 6, 7, 8A, 8B, 9A, 9B</t>
-        </is>
-      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1130,11 +865,6 @@
           <t>151</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>1A, 1B, 1C, 1D, 1E, 1F, 2, 3, 4, 5</t>
-        </is>
-      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1142,11 +872,6 @@
           <t>152</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1154,11 +879,6 @@
           <t>153</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5A, 5B, 5C, 5D1, 5D2, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1166,11 +886,6 @@
           <t>154</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>1, 2, 3A, 3B, 3C</t>
-        </is>
-      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1178,11 +893,6 @@
           <t>155</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6, 7</t>
-        </is>
-      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1190,11 +900,6 @@
           <t>156</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>1, 10, 2, 3, 4, 5, 6, 7, 8, 9A, 9B</t>
-        </is>
-      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1202,11 +907,6 @@
           <t>157</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1214,11 +914,6 @@
           <t>158</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1226,11 +921,6 @@
           <t>159</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>10, 11, 12, 1A1, 1A2, 1A3, 1A4, 1B, 1C, 2A, 2B, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -1238,11 +928,6 @@
           <t>16</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1250,11 +935,6 @@
           <t>160</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>10, 11, 1A, 1B, 2, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1262,11 +942,6 @@
           <t>161</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -1274,11 +949,6 @@
           <t>162</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12A, 12B, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 23, 24, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -1286,11 +956,6 @@
           <t>163</t>
         </is>
       </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5A, 5B, 5C1, 5C2</t>
-        </is>
-      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -1298,11 +963,6 @@
           <t>164</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -1310,11 +970,6 @@
           <t>165</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -1322,11 +977,6 @@
           <t>166</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 2A, 2B, 3, 4A, 4B, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -1334,11 +984,6 @@
           <t>167</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>1A1, 1A2, 1B, 2, 3, 4</t>
-        </is>
-      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -1346,11 +991,6 @@
           <t>168</t>
         </is>
       </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6, 7, 8</t>
-        </is>
-      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -1358,11 +998,6 @@
           <t>169</t>
         </is>
       </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -1370,11 +1005,6 @@
           <t>17</t>
         </is>
       </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -1382,11 +1012,6 @@
           <t>170</t>
         </is>
       </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>1, 2, 3</t>
-        </is>
-      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -1394,11 +1019,6 @@
           <t>171</t>
         </is>
       </c>
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -1406,11 +1026,6 @@
           <t>172</t>
         </is>
       </c>
-      <c r="B83" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -1418,11 +1033,6 @@
           <t>173</t>
         </is>
       </c>
-      <c r="B84" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -1430,11 +1040,6 @@
           <t>174</t>
         </is>
       </c>
-      <c r="B85" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5A, 5B, 5C, 5D, 5E, 6, 7</t>
-        </is>
-      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -1442,11 +1047,6 @@
           <t>175</t>
         </is>
       </c>
-      <c r="B86" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -1454,11 +1054,6 @@
           <t>176</t>
         </is>
       </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6, 7</t>
-        </is>
-      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -1466,11 +1061,6 @@
           <t>177</t>
         </is>
       </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -1478,11 +1068,6 @@
           <t>178</t>
         </is>
       </c>
-      <c r="B89" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -1490,11 +1075,6 @@
           <t>179</t>
         </is>
       </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 23, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -1502,11 +1082,6 @@
           <t>18</t>
         </is>
       </c>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 2, 3, 4A, 4B, 5A, 5B, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -1514,11 +1089,6 @@
           <t>180</t>
         </is>
       </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 23, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -1526,11 +1096,6 @@
           <t>181</t>
         </is>
       </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 1A, 1B, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -1538,11 +1103,6 @@
           <t>182</t>
         </is>
       </c>
-      <c r="B94" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 2, 3, 4, 5A, 5B, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -1550,11 +1110,6 @@
           <t>183</t>
         </is>
       </c>
-      <c r="B95" t="inlineStr">
-        <is>
-          <t>1, 10A, 10B, 10C, 10D, 2A, 2B, 3, 4, 5, 6, 7, 8, 9A, 9B</t>
-        </is>
-      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -1562,11 +1117,6 @@
           <t>184</t>
         </is>
       </c>
-      <c r="B96" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14A, 14B1, 14B2, 14B3, 15, 16, 17, 18, 2, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -1574,11 +1124,6 @@
           <t>185</t>
         </is>
       </c>
-      <c r="B97" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -1586,11 +1131,6 @@
           <t>186</t>
         </is>
       </c>
-      <c r="B98" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 23, 24, 25, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -1598,11 +1138,6 @@
           <t>187</t>
         </is>
       </c>
-      <c r="B99" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 3, 4, 5, 6, 7A1, 7A2, 7B, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -1610,11 +1145,6 @@
           <t>188</t>
         </is>
       </c>
-      <c r="B100" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -1622,11 +1152,6 @@
           <t>189</t>
         </is>
       </c>
-      <c r="B101" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 2, 3, 4, 5, 6, 7A, 7B, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -1634,11 +1159,6 @@
           <t>19</t>
         </is>
       </c>
-      <c r="B102" t="inlineStr">
-        <is>
-          <t>1, 10, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -1646,11 +1166,6 @@
           <t>190</t>
         </is>
       </c>
-      <c r="B103" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -1658,11 +1173,6 @@
           <t>191</t>
         </is>
       </c>
-      <c r="B104" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 2A, 2B, 2C1, 2C2, 3, 4, 5, 6, 7, 8A, 8B, 9</t>
-        </is>
-      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -1670,11 +1180,6 @@
           <t>192</t>
         </is>
       </c>
-      <c r="B105" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -1682,11 +1187,6 @@
           <t>193</t>
         </is>
       </c>
-      <c r="B106" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -1694,11 +1194,6 @@
           <t>194</t>
         </is>
       </c>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>10, 11, 1A, 1B, 2, 3, 4, 5, 6A, 6B, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -1706,11 +1201,6 @@
           <t>195</t>
         </is>
       </c>
-      <c r="B108" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 2, 3, 4, 5, 6A, 6B, 6C, 6D, 6E, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -1718,11 +1208,6 @@
           <t>196</t>
         </is>
       </c>
-      <c r="B109" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -1730,11 +1215,6 @@
           <t>197</t>
         </is>
       </c>
-      <c r="B110" t="inlineStr">
-        <is>
-          <t>1, 10, 11A, 11B, 12, 13, 14, 15, 16, 17, 18, 19, 2, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -1742,11 +1222,6 @@
           <t>198</t>
         </is>
       </c>
-      <c r="B111" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12A, 12B, 12C, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -1754,11 +1229,6 @@
           <t>199</t>
         </is>
       </c>
-      <c r="B112" t="inlineStr">
-        <is>
-          <t>1, 10A, 10B, 2, 3, 4, 5, 6A, 6B, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -1766,11 +1236,6 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B113" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -1778,11 +1243,6 @@
           <t>20</t>
         </is>
       </c>
-      <c r="B114" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 2, 3, 4, 5, 6, 7A, 7B, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -1790,11 +1250,6 @@
           <t>200</t>
         </is>
       </c>
-      <c r="B115" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 3, 4, 5, 6, 7A, 7B, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -1802,11 +1257,6 @@
           <t>201</t>
         </is>
       </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -1814,11 +1264,6 @@
           <t>202</t>
         </is>
       </c>
-      <c r="B117" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 23, 24, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -1826,11 +1271,6 @@
           <t>203</t>
         </is>
       </c>
-      <c r="B118" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -1838,11 +1278,6 @@
           <t>204</t>
         </is>
       </c>
-      <c r="B119" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19A, 19B, 2, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 3, 30, 31, 32A, 32B, 33, 34, 35, 36, 37A, 37B, 37C, 38, 39, 40, 41, 42A, 42B, 43, 4A, 4B, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -1850,11 +1285,6 @@
           <t>205</t>
         </is>
       </c>
-      <c r="B120" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18A, 18B, 19, 2, 20, 21, 22, 23A, 23B, 24, 25, 26, 27, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -1862,11 +1292,6 @@
           <t>206</t>
         </is>
       </c>
-      <c r="B121" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 3, 4, 5, 6, 7, 8, 9A, 9B</t>
-        </is>
-      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -1874,11 +1299,6 @@
           <t>207</t>
         </is>
       </c>
-      <c r="B122" t="inlineStr">
-        <is>
-          <t>1, 10A, 10B, 11, 12, 13, 14, 15, 16, 17, 18, 19A, 19B, 2, 20, 21, 3, 4A, 4B, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -1886,11 +1306,6 @@
           <t>208</t>
         </is>
       </c>
-      <c r="B123" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 2, 3A1A, 3A1B, 3A2A, 3A2B, 3B, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -1898,11 +1313,6 @@
           <t>209</t>
         </is>
       </c>
-      <c r="B124" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 2, 3, 4, 5A1, 5A2, 5B, 6, 7A, 7B1, 7B2, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -1910,11 +1320,6 @@
           <t>21</t>
         </is>
       </c>
-      <c r="B125" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 2, 3, 4, 5A, 5B, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -1922,11 +1327,6 @@
           <t>210</t>
         </is>
       </c>
-      <c r="B126" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16A, 16B, 16C, 17, 18, 19, 2, 20A, 20B, 21, 22, 23, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -1934,11 +1334,6 @@
           <t>211</t>
         </is>
       </c>
-      <c r="B127" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -1946,11 +1341,6 @@
           <t>212</t>
         </is>
       </c>
-      <c r="B128" t="inlineStr">
-        <is>
-          <t>10, 11, 12A, 12B, 13, 1A, 1B, 2A, 2B, 3, 4, 5, 6A, 6B, 6C, 7A, 7B, 7C, 8, 9A, 9B, 9C</t>
-        </is>
-      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -1958,11 +1348,6 @@
           <t>213</t>
         </is>
       </c>
-      <c r="B129" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -1970,11 +1355,6 @@
           <t>214</t>
         </is>
       </c>
-      <c r="B130" t="inlineStr">
-        <is>
-          <t>11, 12, 13, 14, 15, 16, 17, 18, 19, 1A, 2, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 3, 30, 31, 32, 33, 34, 35, 36, 4, 5, 6, 7, 8</t>
-        </is>
-      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -1982,11 +1362,6 @@
           <t>215</t>
         </is>
       </c>
-      <c r="B131" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14A1A1, 14A2, 14B, 14C, 14D, 14E, 14F1A, 14F2, 15, 16, 17, 18, 19A, 19B, 2, 20, 21, 22, 23, 3, 4A1A, 4A1B, 4A1C, 4A2, 4A3, 4A4, 4A5, 4B, 4C, 4D, 5, 6, 7A, 7B, 7C, 7D, 7E, 8, 9A1, 9A2, 9B</t>
-        </is>
-      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -1994,11 +1369,6 @@
           <t>216</t>
         </is>
       </c>
-      <c r="B132" t="inlineStr">
-        <is>
-          <t>1, 10, 2, 3, 4A, 4B, 5, 6, 7, 8A1A1A, 8A1B, 8A1C, 8A2, 8B, 9</t>
-        </is>
-      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -2006,11 +1376,6 @@
           <t>217</t>
         </is>
       </c>
-      <c r="B133" t="inlineStr">
-        <is>
-          <t>1, 10, 11A, 11B, 11C, 12A, 12B, 2A, 2B, 2C, 2D, 2E, 2F, 3, 4A, 4B, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -2018,11 +1383,6 @@
           <t>218</t>
         </is>
       </c>
-      <c r="B134" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2A, 2B1, 2B2</t>
-        </is>
-      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -2030,11 +1390,6 @@
           <t>219</t>
         </is>
       </c>
-      <c r="B135" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6, 7A1, 7A2, 7B, 7C, 7D, 7E, 7F, 7G, 8</t>
-        </is>
-      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -2042,11 +1397,6 @@
           <t>22</t>
         </is>
       </c>
-      <c r="B136" t="inlineStr">
-        <is>
-          <t>1, 10, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -2054,11 +1404,6 @@
           <t>220</t>
         </is>
       </c>
-      <c r="B137" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13A, 13B, 14, 15, 16, 17A, 17B, 17C, 17D, 18A, 18B, 19A, 19B, 2, 20, 21, 22A1, 22A2, 22B, 23, 24, 25, 26, 27A, 27B, 27C, 28A, 28B, 28C, 3A, 3B, 3C1, 3C2, 3D1, 3D2A, 3D2B, 3E, 3F, 4A, 4B, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -2066,11 +1411,6 @@
           <t>221</t>
         </is>
       </c>
-      <c r="B138" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 23, 3, 4, 5, 6, 7A, 7B, 7C, 7D, 7E, 7F, 7G, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -2078,11 +1418,6 @@
           <t>222</t>
         </is>
       </c>
-      <c r="B139" t="inlineStr">
-        <is>
-          <t>10, 11, 12A, 12B, 13A, 13B, 14A, 14B, 15, 16, 17A, 17B, 18, 19, 1A, 1B, 2, 20, 21, 22, 3, 4, 5A, 5B, 6A, 6B, 7A, 7B, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -2090,11 +1425,6 @@
           <t>223</t>
         </is>
       </c>
-      <c r="B140" t="inlineStr">
-        <is>
-          <t>1, 10A, 10B, 10C, 10D, 11A, 11B, 12, 13A, 13B, 13C, 13D, 13E, 13F, 14A, 14B, 15A, 15B, 16A, 16B, 2A, 2B, 3A1, 3A2, 3B, 4A, 4B, 5, 6A, 6B, 7, 8, 9A, 9B, 9C, 9D</t>
-        </is>
-      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -2102,11 +1432,6 @@
           <t>224</t>
         </is>
       </c>
-      <c r="B141" t="inlineStr">
-        <is>
-          <t>1, 10A1A1A1A, 10A1B, 10A1C, 10A1D, 10A1E, 10A2, 10A3, 10B, 11, 12, 13A, 13B, 14, 15, 16, 17, 18, 2, 3A, 3B, 4, 5, 6, 7A, 7B, 8, 9A, 9B</t>
-        </is>
-      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -2114,11 +1439,6 @@
           <t>225</t>
         </is>
       </c>
-      <c r="B142" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12A1A1, 12A1B, 12A2, 12B, 13A, 13B, 13C, 13D, 13E, 14A1A, 14A1B, 14A2, 14B, 14C1, 14C2, 14C3, 15A1A, 15A2, 15B, 16A1A, 16A1B, 16A2, 16B, 17, 18, 2A1, 2A2, 2B, 3, 4A, 4B, 4C, 4D, 5A, 5B, 6A, 6B, 6C1, 6C2, 6D, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -2126,11 +1446,6 @@
           <t>226</t>
         </is>
       </c>
-      <c r="B143" t="inlineStr">
-        <is>
-          <t>1A1, 1A2, 1B, 2A, 2B1A, 2B1B, 2B2, 3, 4, 5, 6</t>
-        </is>
-      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -2138,11 +1453,6 @@
           <t>227</t>
         </is>
       </c>
-      <c r="B144" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2, 3, 4, 5, 6</t>
-        </is>
-      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -2150,11 +1460,6 @@
           <t>228</t>
         </is>
       </c>
-      <c r="B145" t="inlineStr">
-        <is>
-          <t>1A, 1B, 1C, 1D, 1E, 1F, 1G, 1H, 1I, 1J, 1K, 2, 3, 4, 5, 6A, 6B, 7</t>
-        </is>
-      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -2162,11 +1467,6 @@
           <t>229</t>
         </is>
       </c>
-      <c r="B146" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -2174,11 +1474,6 @@
           <t>23</t>
         </is>
       </c>
-      <c r="B147" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6, 7, 8A, 8B</t>
-        </is>
-      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -2186,11 +1481,6 @@
           <t>230</t>
         </is>
       </c>
-      <c r="B148" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -2198,11 +1488,6 @@
           <t>231</t>
         </is>
       </c>
-      <c r="B149" t="inlineStr">
-        <is>
-          <t>10, 11, 12, 13, 1A, 1B, 2, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -2210,11 +1495,6 @@
           <t>232</t>
         </is>
       </c>
-      <c r="B150" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -2222,11 +1502,6 @@
           <t>233</t>
         </is>
       </c>
-      <c r="B151" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12A, 12B, 13A, 13B, 13C, 14, 2, 3, 4, 5A, 5B, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -2234,11 +1509,6 @@
           <t>234</t>
         </is>
       </c>
-      <c r="B152" t="inlineStr">
-        <is>
-          <t>10, 11, 1A, 1B, 1C, 2, 3, 4, 5, 6A, 6B, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -2246,11 +1516,6 @@
           <t>235</t>
         </is>
       </c>
-      <c r="B153" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 3, 4, 5, 6, 7, 8A, 8B</t>
-        </is>
-      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -2258,11 +1523,6 @@
           <t>236</t>
         </is>
       </c>
-      <c r="B154" t="inlineStr">
-        <is>
-          <t>1, 2, 3</t>
-        </is>
-      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -2270,11 +1530,6 @@
           <t>237</t>
         </is>
       </c>
-      <c r="B155" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -2282,11 +1537,6 @@
           <t>238</t>
         </is>
       </c>
-      <c r="B156" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -2294,11 +1544,6 @@
           <t>239</t>
         </is>
       </c>
-      <c r="B157" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2A, 2B, 2C, 3A, 3B, 3C, 3D, 3E, 3F, 3G, 3H, 3I, 3J, 3K, 3L, 3M, 3N, 3O, 3P, 3Q, 3R, 3S, 3T, 3U, 3V, 3W, 3X, 4A, 4B, 5A, 5B, 5C, 6A, 6B, 6C, 6D, 6E, 6F, 6G, 7, 8, 9A, 9B, 9C</t>
-        </is>
-      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -2306,11 +1551,6 @@
           <t>24</t>
         </is>
       </c>
-      <c r="B158" t="inlineStr">
-        <is>
-          <t>1, 10A1, 10A2, 10A3, 10B, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -2318,11 +1558,6 @@
           <t>240</t>
         </is>
       </c>
-      <c r="B159" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 2C, 2D, 2E, 2F, 2G, 2H, 2I, 3A, 3B, 3C, 3D, 3E, 3F, 4, 5, 6, 7, 8A, 8B, 9</t>
-        </is>
-      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -2330,11 +1565,6 @@
           <t>241</t>
         </is>
       </c>
-      <c r="B160" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -2342,11 +1572,6 @@
           <t>242</t>
         </is>
       </c>
-      <c r="B161" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4</t>
-        </is>
-      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -2354,11 +1579,6 @@
           <t>243</t>
         </is>
       </c>
-      <c r="B162" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -2366,11 +1586,6 @@
           <t>244</t>
         </is>
       </c>
-      <c r="B163" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -2378,11 +1593,6 @@
           <t>245</t>
         </is>
       </c>
-      <c r="B164" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -2390,11 +1600,6 @@
           <t>246</t>
         </is>
       </c>
-      <c r="B165" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -2402,11 +1607,6 @@
           <t>247</t>
         </is>
       </c>
-      <c r="B166" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -2414,11 +1614,6 @@
           <t>248</t>
         </is>
       </c>
-      <c r="B167" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4A1, 4A2, 4B, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -2426,11 +1621,6 @@
           <t>249</t>
         </is>
       </c>
-      <c r="B168" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 2C, 2D, 3A, 3B, 3C, 3D, 3E, 3F, 4, 5A, 5B, 5C, 6A, 6B, 7A, 7B, 8A, 8B, 9A, 9B, 9C1, 9C2A, 9C2B</t>
-        </is>
-      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -2438,11 +1628,6 @@
           <t>25</t>
         </is>
       </c>
-      <c r="B169" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15A, 15B, 16, 17, 18A1A, 18A1B, 18A2, 18B, 19, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -2450,11 +1635,6 @@
           <t>250</t>
         </is>
       </c>
-      <c r="B170" t="inlineStr">
-        <is>
-          <t>1, 10A, 10B, 11, 2, 3A, 3B, 3C, 4, 5, 6A, 6B, 6C, 7A, 7B, 8A, 8B1, 8B2, 9A, 9B, 9C</t>
-        </is>
-      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -2462,11 +1642,6 @@
           <t>251</t>
         </is>
       </c>
-      <c r="B171" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13A, 13B, 14A1A, 14A1B, 14A2, 14B, 15A, 15B, 15C, 16A, 16B, 17A1, 17A2, 17B, 18A1, 18A2, 18B, 18C, 19, 20A, 20B, 21A, 21B, 2A, 2B, 3A, 3B, 3C, 4A, 4B, 5A1, 5A2, 5A3, 5B, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -2474,11 +1649,6 @@
           <t>252</t>
         </is>
       </c>
-      <c r="B172" t="inlineStr">
-        <is>
-          <t>1A, 1B1, 1B2, 2A, 2B, 3, 4, 5A, 5B, 6</t>
-        </is>
-      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -2486,11 +1656,6 @@
           <t>253</t>
         </is>
       </c>
-      <c r="B173" t="inlineStr">
-        <is>
-          <t>10, 11A, 11B, 11C, 12, 13, 1A, 1B, 1C, 2A, 2B, 2C, 3, 4, 5, 6, 7, 8A, 8B, 8C, 8D, 9A, 9B, 9C</t>
-        </is>
-      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -2498,11 +1663,6 @@
           <t>254</t>
         </is>
       </c>
-      <c r="B174" t="inlineStr">
-        <is>
-          <t>1, 10, 11A, 11B, 11C, 11D, 11E, 11F, 11G, 11H, 11I, 12, 13, 14A, 14B, 15A, 15B, 15C, 16A, 16B, 2A1, 2A2, 2B, 3, 4, 5A, 5B, 6A, 6B, 7A, 7B, 8, 9A, 9B</t>
-        </is>
-      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -2510,11 +1670,6 @@
           <t>255</t>
         </is>
       </c>
-      <c r="B175" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13A, 13B1A1, 13B1A2, 13B1A3, 13B1B, 13B2, 13C, 13D1, 13D2, 14, 15A1A, 15A1B, 15A2A, 15A2B, 15B, 16, 17A, 17B1, 17B2A, 17B2B, 18, 19, 2, 20, 21, 22, 23A, 23B, 23C, 24, 3, 4, 5A, 5B1, 5B2, 5C, 5D1A, 5D1B, 5D2, 6, 7A1, 7A2A, 7A2B, 7B, 8A, 8B, 9</t>
-        </is>
-      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -2522,11 +1677,6 @@
           <t>256</t>
         </is>
       </c>
-      <c r="B176" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -2534,11 +1684,6 @@
           <t>257</t>
         </is>
       </c>
-      <c r="B177" t="inlineStr">
-        <is>
-          <t>1, 10A, 10B, 11, 12, 2A, 2B, 2C, 2D, 2E, 2F, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -2546,11 +1691,6 @@
           <t>258</t>
         </is>
       </c>
-      <c r="B178" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -2558,11 +1698,6 @@
           <t>259</t>
         </is>
       </c>
-      <c r="B179" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 2C, 3, 4A, 4B, 4C, 5, 6, 7A, 7B</t>
-        </is>
-      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -2570,11 +1705,6 @@
           <t>26</t>
         </is>
       </c>
-      <c r="B180" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -2582,11 +1712,6 @@
           <t>260</t>
         </is>
       </c>
-      <c r="B181" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 23A, 23B, 24, 25, 26, 27, 28, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -2594,11 +1719,6 @@
           <t>261</t>
         </is>
       </c>
-      <c r="B182" t="inlineStr">
-        <is>
-          <t>10, 11, 12, 13, 14, 1A, 1B, 1C, 1D, 1E, 2, 3, 4, 5, 6A, 6B, 6C, 6D, 7, 8A, 8B, 9</t>
-        </is>
-      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -2606,11 +1726,6 @@
           <t>262</t>
         </is>
       </c>
-      <c r="B183" t="inlineStr">
-        <is>
-          <t>10, 11A, 11B, 11C, 11D, 12, 1A, 1B, 1C, 1D, 2A, 2B, 3, 4, 5, 6, 7, 8A, 8B, 9A, 9B, 9C</t>
-        </is>
-      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -2618,11 +1733,6 @@
           <t>263</t>
         </is>
       </c>
-      <c r="B184" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 2, 3, 4, 5, 6, 7A1, 7A2, 7B, 8A, 8B, 9A, 9B</t>
-        </is>
-      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -2630,11 +1740,6 @@
           <t>264</t>
         </is>
       </c>
-      <c r="B185" t="inlineStr">
-        <is>
-          <t>10, 11, 1A, 1B, 2A, 2B, 2C1, 2C2, 3A, 3B, 4A, 4B, 5A, 5B, 5C, 5D, 5E, 5F, 5G, 6, 7A, 7B, 7C, 7D, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -2642,11 +1747,6 @@
           <t>265</t>
         </is>
       </c>
-      <c r="B186" t="inlineStr">
-        <is>
-          <t>10, 11, 12, 13, 14, 15, 16, 17, 18A, 18B, 19A, 19B, 1A, 1B, 20, 21A, 21B, 22, 23A, 23B, 24, 25, 2A, 2B, 3, 4, 5, 6A, 6B, 7A, 7B, 8A, 8B, 9</t>
-        </is>
-      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -2654,11 +1754,6 @@
           <t>266</t>
         </is>
       </c>
-      <c r="B187" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 2A, 2B, 3A, 3B, 4, 5A, 5B, 5C, 5D, 6A, 6B, 7, 8, 9A, 9B, 9C1, 9C2, 9C3</t>
-        </is>
-      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -2666,11 +1761,6 @@
           <t>267</t>
         </is>
       </c>
-      <c r="B188" t="inlineStr">
-        <is>
-          <t>10A, 10B, 10C, 10D, 11A, 11B, 11C, 12, 13, 14, 15, 16, 17, 18, 19, 1A, 1B, 1C1, 1C2, 2, 20, 21A1, 21A2, 21B, 21C, 21D, 3, 4A, 4B, 5A, 5B, 6, 7A, 7B, 8A, 8B, 9A, 9B</t>
-        </is>
-      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -2678,11 +1768,6 @@
           <t>268</t>
         </is>
       </c>
-      <c r="B189" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13A, 13B, 14A1, 14A2, 14B, 14C, 15, 16, 17A, 17B, 18A, 18B, 19A, 19B, 2, 20, 21, 22, 23, 24, 3, 4A, 4B, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -2690,11 +1775,6 @@
           <t>269</t>
         </is>
       </c>
-      <c r="B190" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12A1, 12A2, 12B1, 12B2, 13, 14, 15A1, 15A2, 15B, 16, 17, 18, 19, 20, 21A1A, 21A1B1, 21B, 22, 23, 24, 25, 26, 27, 2A, 2B, 3A, 3B, 3C, 4, 5, 6, 7, 8A1, 8A2, 8B, 9A, 9B</t>
-        </is>
-      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -2702,11 +1782,6 @@
           <t>27</t>
         </is>
       </c>
-      <c r="B191" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -2714,11 +1789,6 @@
           <t>270</t>
         </is>
       </c>
-      <c r="B192" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12A, 12B, 12C, 12D, 12E, 13A, 13B, 13C, 14A, 14B, 15A, 15B, 15C, 15D, 15E, 15F, 15G, 2, 3A, 3B, 4, 5, 6A, 6B, 6C, 6D, 7, 8, 9A, 9B, 9C, 9D</t>
-        </is>
-      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -2726,11 +1796,6 @@
           <t>271</t>
         </is>
       </c>
-      <c r="B193" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4</t>
-        </is>
-      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -2738,11 +1803,6 @@
           <t>272</t>
         </is>
       </c>
-      <c r="B194" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13A1, 13A2, 13A3, 13A4, 13B, 13C, 13D, 13E, 13F, 14, 15A1, 15A2, 15B, 15C, 16A, 16B, 17A, 17B, 18A, 18B, 19, 201A1, 201A2, 20A, 20B1A, 20B1B, 20B1C, 20B1D, 20B2, 20C1, 20C2, 20D, 20E, 20F, 20G1, 20G2, 20G3, 20G4, 20G5, 20G6, 20G7, 20H1, 20H2, 20H3, 20H4, 20H5, 20H6, 20IB, 20J, 20K, 20L, 21A1, 21A2, 21A3, 21A4, 21A5, 21A6, 21A7, 21B, 22, 23A, 23B1, 23B2, 2A, 2B, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -2750,11 +1810,6 @@
           <t>273</t>
         </is>
       </c>
-      <c r="B195" t="inlineStr">
-        <is>
-          <t>10, 11, 12, 13A, 13B, 13C, 13D, 13E, 14, 15, 16, 17A, 17B, 17C, 17D, 1A, 1B, 2A, 2B, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -2762,11 +1817,6 @@
           <t>274</t>
         </is>
       </c>
-      <c r="B196" t="inlineStr">
-        <is>
-          <t>10, 11, 12, 13, 14, 1A, 1B, 1C, 1D, 1E, 1F, 1G, 2, 3, 4, 5, 6, 7A, 7B, 7C, 7D, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -2774,11 +1824,6 @@
           <t>275</t>
         </is>
       </c>
-      <c r="B197" t="inlineStr">
-        <is>
-          <t>1, 10, 11A, 11B1, 11B2, 12, 13, 14, 15A, 15B, 16, 17, 18A, 18B, 19A1, 19A2, 19A3, 19B1, 19B2, 19B3, 2, 20A, 20B1A1, 20B1A2, 20B2, 21, 3A, 3B, 3C, 4, 5, 6, 7, 8A, 8B, 9</t>
-        </is>
-      </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -2786,11 +1831,6 @@
           <t>276</t>
         </is>
       </c>
-      <c r="B198" t="inlineStr">
-        <is>
-          <t>10A, 10B1, 10B2, 10C, 11, 1A, 1B, 1C, 1D, 1E, 2, 3, 4, 5A, 5B1, 5B2, 6A, 6B, 7, 8A, 8B, 9A, 9B</t>
-        </is>
-      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -2798,11 +1838,6 @@
           <t>277</t>
         </is>
       </c>
-      <c r="B199" t="inlineStr">
-        <is>
-          <t>1, 10A, 10B, 11, 2, 3, 4A, 4B, 5, 6A, 6B, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -2810,11 +1845,6 @@
           <t>278</t>
         </is>
       </c>
-      <c r="B200" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 2A, 2B, 3, 4, 5, 6, 7A, 7B, 8, 9A, 9B</t>
-        </is>
-      </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -2822,11 +1852,6 @@
           <t>279</t>
         </is>
       </c>
-      <c r="B201" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 2, 3A1, 3A2, 3A3, 3B, 3C, 4, 5, 6A1, 6A2, 6B, 7, 8A, 8B, 8C, 8D, 9</t>
-        </is>
-      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -2834,11 +1859,6 @@
           <t>28</t>
         </is>
       </c>
-      <c r="B202" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -2846,11 +1866,6 @@
           <t>280</t>
         </is>
       </c>
-      <c r="B203" t="inlineStr">
-        <is>
-          <t>10A, 10B, 11A, 11B, 12, 13, 14A, 14B, 15, 16A, 16B, 16C, 17, 18A, 18B1, 18B2, 18C, 19A1, 19A2, 19A3, 19B, 1A1, 1A2, 1A3, 1B, 2, 20, 21, 3A1, 3A2, 3B1, 3B2, 3B3, 4, 5A, 5B, 6, 7A, 7B, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -2858,11 +1873,6 @@
           <t>281</t>
         </is>
       </c>
-      <c r="B204" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15A, 15B1, 15B2, 15B3, 16, 17, 2A, 2B, 3A, 3B, 3C, 4A, 4B, 4C, 5A, 5B, 6, 7A, 7B1, 7B2, 7B3, 7C, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -2870,11 +1880,6 @@
           <t>282</t>
         </is>
       </c>
-      <c r="B205" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -2882,11 +1887,6 @@
           <t>283</t>
         </is>
       </c>
-      <c r="B206" t="inlineStr">
-        <is>
-          <t>1, 2, 3</t>
-        </is>
-      </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -2894,11 +1894,6 @@
           <t>284</t>
         </is>
       </c>
-      <c r="B207" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -2906,11 +1901,6 @@
           <t>285</t>
         </is>
       </c>
-      <c r="B208" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -2918,11 +1908,6 @@
           <t>286</t>
         </is>
       </c>
-      <c r="B209" t="inlineStr">
-        <is>
-          <t>1, 10, 2A, 2B, 3, 4A, 4B2, 5, 6, 7, 8, 9, 9A</t>
-        </is>
-      </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -2930,11 +1915,6 @@
           <t>287</t>
         </is>
       </c>
-      <c r="B210" t="inlineStr">
-        <is>
-          <t>1, 100A, 100B, 100C, 10A, 10B, 11, 12, 13, 14, 15, 16, 17A, 17B, 17C, 17D, 17E, 18, 19, 2, 20, 21, 22A1, 22A2, 22B, 23A, 23B, 23C, 24, 25A, 25B, 26, 27A, 27B, 27C1, 27C2, 27C3, 27D, 27E, 28A, 28B, 29A, 29B, 3, 30, 31, 32, 33A, 33B, 33C, 34, 35, 36, 37, 38, 39, 4, 40A, 40B, 40C, 41, 42, 43, 44, 45A, 45B1, 45B2, 46, 47A, 47B, 48, 49A, 49B, 50A1, 50A2, 50B1, 50B2, 51, 52, 53, 54, 55, 56A, 56B, 57, 58, 59, 5A, 5B, 5C, 6, 60A, 60B, 61, 62A, 62B, 63, 64A, 64B, 65, 66, 67, 68, 69, 7, 70, 71, 72A1, 72A2, 72B1, 72B2, 72B3, 73, 74A, 74B, 75A1, 75A2, 75B, 76, 77A, 77B, 78, 79, 80, 81, 82, 83, 84, 85, 86, 87A, 87B, 88, 89A, 89B, 8A, 8B1, 8B2, 90, 91, 92, 93, 94, 95, 96A, 96B, 96C, 96D, 97, 98, 99, 9A, 9B</t>
-        </is>
-      </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -2942,11 +1922,6 @@
           <t>288</t>
         </is>
       </c>
-      <c r="B211" t="inlineStr">
-        <is>
-          <t>1, 2, 3A, 3B, 3C, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -2954,11 +1929,6 @@
           <t>289</t>
         </is>
       </c>
-      <c r="B212" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -2966,11 +1936,6 @@
           <t>29</t>
         </is>
       </c>
-      <c r="B213" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -2978,11 +1943,6 @@
           <t>290</t>
         </is>
       </c>
-      <c r="B214" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -2990,11 +1950,6 @@
           <t>291</t>
         </is>
       </c>
-      <c r="B215" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -3002,11 +1957,6 @@
           <t>292</t>
         </is>
       </c>
-      <c r="B216" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 3, 4, 5A, 5B, 6</t>
-        </is>
-      </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -3014,11 +1964,6 @@
           <t>293</t>
         </is>
       </c>
-      <c r="B217" t="inlineStr">
-        <is>
-          <t>1, 2, 3</t>
-        </is>
-      </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -3026,11 +1971,6 @@
           <t>294</t>
         </is>
       </c>
-      <c r="B218" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
-      </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -3038,11 +1978,6 @@
           <t>295</t>
         </is>
       </c>
-      <c r="B219" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4A, 4B, 4C, 4D, 5A, 5B, 5C, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -3050,11 +1985,6 @@
           <t>296</t>
         </is>
       </c>
-      <c r="B220" t="inlineStr">
-        <is>
-          <t>1, 10A, 10B, 10C, 10D, 2, 3, 4, 5, 6, 7A, 7B, 7C, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -3062,11 +1992,6 @@
           <t>297</t>
         </is>
       </c>
-      <c r="B221" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6, 7, 8</t>
-        </is>
-      </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -3074,11 +1999,6 @@
           <t>298</t>
         </is>
       </c>
-      <c r="B222" t="inlineStr">
-        <is>
-          <t>1, 2, 3A, 3B, 3C, 4, 5A, 5B</t>
-        </is>
-      </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -3086,11 +2006,6 @@
           <t>299</t>
         </is>
       </c>
-      <c r="B223" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4A, 4B, 5</t>
-        </is>
-      </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -3098,11 +2013,6 @@
           <t>3</t>
         </is>
       </c>
-      <c r="B224" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -3110,11 +2020,6 @@
           <t>30</t>
         </is>
       </c>
-      <c r="B225" t="inlineStr">
-        <is>
-          <t>1, 10A, 10B, 11, 12, 13, 14, 15, 16, 17, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -3122,11 +2027,6 @@
           <t>300</t>
         </is>
       </c>
-      <c r="B226" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -3134,11 +2034,6 @@
           <t>301</t>
         </is>
       </c>
-      <c r="B227" t="inlineStr">
-        <is>
-          <t>1, 10A, 10B, 11, 12, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -3146,11 +2041,6 @@
           <t>302</t>
         </is>
       </c>
-      <c r="B228" t="inlineStr">
-        <is>
-          <t>10, 11, 12, 13, 1A, 1B, 1C, 2, 3A, 3B, 4A, 4B, 5A, 5B, 6A, 6B, 7A, 7B, 7C, 8A, 8B, 8C, 9</t>
-        </is>
-      </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -3158,11 +2048,6 @@
           <t>303</t>
         </is>
       </c>
-      <c r="B229" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -3170,11 +2055,6 @@
           <t>304</t>
         </is>
       </c>
-      <c r="B230" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6, 7</t>
-        </is>
-      </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -3182,11 +2062,6 @@
           <t>305</t>
         </is>
       </c>
-      <c r="B231" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6, 7, 8, 9A, 9B</t>
-        </is>
-      </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -3194,11 +2069,6 @@
           <t>306</t>
         </is>
       </c>
-      <c r="B232" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4A, 4B, 5, 6</t>
-        </is>
-      </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -3206,11 +2076,6 @@
           <t>307</t>
         </is>
       </c>
-      <c r="B233" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2A1, 2A2, 2A3, 2A4, 2B, 3A, 3B, 3C1A, 3C1B, 3C2, 4A, 4B, 5A, 5B1, 5B2, 6A1, 6A2, 6A3, 6B, 7A1, 7A2, 7B1, 7B2, 7C1, 7C2, 8A, 8B, 8C</t>
-        </is>
-      </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -3218,11 +2083,6 @@
           <t>308</t>
         </is>
       </c>
-      <c r="B234" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2A, 2B1, 2B2, 3A, 3B1A, 3B2, 4A, 4B, 5A, 5B, 6A, 6B, 7</t>
-        </is>
-      </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -3230,11 +2090,6 @@
           <t>309</t>
         </is>
       </c>
-      <c r="B235" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2A, 2B, 3A1, 3A2, 3B, 4A1, 4A2, 4B1, 4B2, 5A, 5B, 5C, 5D, 6A1A, 6A1B, 6A2A, 6A2B, 6B1A, 6B1B, 6B2, 6C1, 6C2, 6C3, 6D1A1, 6D1A2, 6D2, 6E1, 6E2, 6E3, 6F, 6G, 7</t>
-        </is>
-      </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -3242,11 +2097,6 @@
           <t>31</t>
         </is>
       </c>
-      <c r="B236" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6, 7</t>
-        </is>
-      </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -3254,11 +2104,6 @@
           <t>310</t>
         </is>
       </c>
-      <c r="B237" t="inlineStr">
-        <is>
-          <t>1A, 1B, 1C, 1D, 1E, 2, 3, 4A, 4B, 5</t>
-        </is>
-      </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -3266,11 +2111,6 @@
           <t>311</t>
         </is>
       </c>
-      <c r="B238" t="inlineStr">
-        <is>
-          <t>1A, 1B, 1C, 1D, 1E, 2A, 2B, 2C, 2D, 2E, 2F, 2G, 2H, 2I, 3</t>
-        </is>
-      </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -3278,11 +2118,6 @@
           <t>312</t>
         </is>
       </c>
-      <c r="B239" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2A, 2B, 2C, 3A, 3B, 3C, 3D, 3E, 3F, 4, 5, 6, 7, 8</t>
-        </is>
-      </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -3290,11 +2125,6 @@
           <t>313</t>
         </is>
       </c>
-      <c r="B240" t="inlineStr">
-        <is>
-          <t>1A1, 1A2, 1B1, 1B2, 2A, 2B, 3A, 3B, 3C, 4A1, 4A2, 4B, 4C, 5A1A, 5A1B, 5A2, 5B, 5C, 6A, 6B, 7, 8A, 8B, 8C, 8D, 9</t>
-        </is>
-      </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -3302,11 +2132,6 @@
           <t>314</t>
         </is>
       </c>
-      <c r="B241" t="inlineStr">
-        <is>
-          <t>1, 2, 3A, 3B, 4A, 4B1, 4B2, 4C1, 4C2, 4D, 4E, 4F, 4G, 4H, 4I, 4J, 5A, 5B, 5C, 5D, 6, 7A, 7B, 7C, 7D1, 7D2</t>
-        </is>
-      </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -3314,11 +2139,6 @@
           <t>315</t>
         </is>
       </c>
-      <c r="B242" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2, 3A, 3B, 4A, 4B, 5A, 5B, 6, 7A, 7B, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -3326,11 +2146,6 @@
           <t>316</t>
         </is>
       </c>
-      <c r="B243" t="inlineStr">
-        <is>
-          <t>1, 10A, 10B, 11A, 11B, 11C, 2A1, 2A2, 2B, 3A, 3B, 4A, 4B1, 4B2, 5A1, 5A2, 5A3, 5B, 6, 7, 8, 9A, 9B</t>
-        </is>
-      </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -3338,11 +2153,6 @@
           <t>317</t>
         </is>
       </c>
-      <c r="B244" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12A, 12B1, 12B2, 13, 14, 2, 3, 4, 5, 6, 7, 8A, 8B, 9A, 9B, 9C</t>
-        </is>
-      </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -3350,11 +2160,6 @@
           <t>318</t>
         </is>
       </c>
-      <c r="B245" t="inlineStr">
-        <is>
-          <t>1A, 1B1, 1B2, 1C1, 1C2, 2, 3, 4, 5A, 5B, 5C, 5D, 5E, 5F, 6, 7, 8</t>
-        </is>
-      </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -3362,11 +2167,6 @@
           <t>319</t>
         </is>
       </c>
-      <c r="B246" t="inlineStr">
-        <is>
-          <t>1, 10A, 10B, 11, 12, 13A, 13B, 2, 3, 4, 5, 6A, 6B, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -3374,11 +2174,6 @@
           <t>32</t>
         </is>
       </c>
-      <c r="B247" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 2, 3, 4A, 4B, 4C, 4D, 5, 6A, 6B, 7, 8A, 8B, 9</t>
-        </is>
-      </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -3386,11 +2181,6 @@
           <t>320</t>
         </is>
       </c>
-      <c r="B248" t="inlineStr">
-        <is>
-          <t>1, 10, 11A, 11B, 12A, 12B, 13, 14, 15, 16, 2, 3, 4A, 4B, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -3398,11 +2188,6 @@
           <t>321</t>
         </is>
       </c>
-      <c r="B249" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 2C, 2D, 2E, 3, 4, 5</t>
-        </is>
-      </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -3410,11 +2195,6 @@
           <t>322</t>
         </is>
       </c>
-      <c r="B250" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15A, 15B, 2, 3, 4A, 4B, 4C, 4D, 4E, 4F, 4G, 5A, 5B, 5C, 5D, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -3422,11 +2202,6 @@
           <t>323</t>
         </is>
       </c>
-      <c r="B251" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -3434,11 +2209,6 @@
           <t>324</t>
         </is>
       </c>
-      <c r="B252" t="inlineStr">
-        <is>
-          <t>1, 2, 3A, 3B, 4, 5, 6, 7, 8A, 8B, 8C, 8D, 8E, 8F, 8G, 9</t>
-        </is>
-      </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -3446,11 +2216,6 @@
           <t>325</t>
         </is>
       </c>
-      <c r="B253" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6, 7, 8</t>
-        </is>
-      </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -3458,11 +2223,6 @@
           <t>326</t>
         </is>
       </c>
-      <c r="B254" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13A, 13B, 14, 15, 16, 17, 18, 19, 2, 3, 4, 5, 6A, 6B, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -3470,11 +2230,6 @@
           <t>327</t>
         </is>
       </c>
-      <c r="B255" t="inlineStr">
-        <is>
-          <t>1, 10, 11A, 11B1, 11B2, 11B3, 12, 13, 14, 15, 16, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -3482,11 +2237,6 @@
           <t>328</t>
         </is>
       </c>
-      <c r="B256" t="inlineStr">
-        <is>
-          <t>1A, 1B1, 1B2, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -3494,11 +2244,6 @@
           <t>329</t>
         </is>
       </c>
-      <c r="B257" t="inlineStr">
-        <is>
-          <t>1, 10A, 10B, 2, 3, 4, 5, 6A, 6B, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -3506,11 +2251,6 @@
           <t>33</t>
         </is>
       </c>
-      <c r="B258" t="inlineStr">
-        <is>
-          <t>1, 2, 3A, 3B, 4A, 4B, 4C, 5A, 5B, 5C1, 5C2, 5D, 6, 7, 8A, 8B</t>
-        </is>
-      </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -3518,11 +2258,6 @@
           <t>330</t>
         </is>
       </c>
-      <c r="B259" t="inlineStr">
-        <is>
-          <t>1A, 1B, 1C, 2A, 2B, 2C, 3A, 3B, 4A1, 4A2, 4B1, 4B2</t>
-        </is>
-      </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -3530,11 +2265,6 @@
           <t>331</t>
         </is>
       </c>
-      <c r="B260" t="inlineStr">
-        <is>
-          <t>1A, 1B, 1C, 2A, 2B, 3, 4, 5A, 5B</t>
-        </is>
-      </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -3542,11 +2272,6 @@
           <t>332</t>
         </is>
       </c>
-      <c r="B261" t="inlineStr">
-        <is>
-          <t>1A, 1B, 1C, 1D1, 1D2, 2, 3A, 3B, 4A, 4B, 5, 6, 7, 8</t>
-        </is>
-      </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -3554,11 +2279,6 @@
           <t>333</t>
         </is>
       </c>
-      <c r="B262" t="inlineStr">
-        <is>
-          <t>1, 10, 11A, 11B, 12, 13, 14, 2A, 2B1, 2B2, 3A, 3B, 4A, 4B, 5, 6A, 6B, 6C, 7A1, 7A2, 7A3, 7B, 8A, 8B, 9A, 9B</t>
-        </is>
-      </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -3566,11 +2286,6 @@
           <t>334</t>
         </is>
       </c>
-      <c r="B263" t="inlineStr">
-        <is>
-          <t>10, 1A, 1B, 2A, 2B, 3, 4, 5, 6, 7A, 7B, 8A, 8B, 9</t>
-        </is>
-      </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -3578,11 +2293,6 @@
           <t>335</t>
         </is>
       </c>
-      <c r="B264" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -3590,11 +2300,6 @@
           <t>336</t>
         </is>
       </c>
-      <c r="B265" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -3602,11 +2307,6 @@
           <t>337</t>
         </is>
       </c>
-      <c r="B266" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6, 7A, 7B, 7C, 7D, 7E, 8</t>
-        </is>
-      </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -3614,11 +2314,6 @@
           <t>338</t>
         </is>
       </c>
-      <c r="B267" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
-      </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -3626,11 +2321,6 @@
           <t>339</t>
         </is>
       </c>
-      <c r="B268" t="inlineStr">
-        <is>
-          <t>1, 10, 2A, 2B, 3A, 3B, 3C, 3D, 3E, 3F, 3G, 3H, 3I, 3J, 4, 5, 6, 7, 8A, 8B, 9</t>
-        </is>
-      </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -3638,11 +2328,6 @@
           <t>34</t>
         </is>
       </c>
-      <c r="B269" t="inlineStr">
-        <is>
-          <t>1, 10A, 10B, 10C, 11, 12, 13A, 13B, 2, 3, 4A, 4B, 4C, 5, 6A, 6B, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -3650,11 +2335,6 @@
           <t>340</t>
         </is>
       </c>
-      <c r="B270" t="inlineStr">
-        <is>
-          <t>1, 10, 11A, 11B, 12A, 12B, 13A, 13B, 14, 2, 3, 4, 5A, 5B, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -3662,11 +2342,6 @@
           <t>341</t>
         </is>
       </c>
-      <c r="B271" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2, 3A1, 3A2, 3B, 4, 5A1, 5A2, 5B1, 5B2, 5C, 5D, 6, 7, 8A1, 8A2, 8A3, 8B</t>
-        </is>
-      </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -3674,11 +2349,6 @@
           <t>342</t>
         </is>
       </c>
-      <c r="B272" t="inlineStr">
-        <is>
-          <t>1, 10, 2A, 2B, 3, 4, 5A, 5B, 6A, 6B, 7A, 7B, 8A, 8B, 9A, 9B</t>
-        </is>
-      </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -3686,11 +2356,6 @@
           <t>343</t>
         </is>
       </c>
-      <c r="B273" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12A1, 12A2, 12B, 13, 2, 3, 4A1, 4A2, 4B, 5A, 5B, 6A, 6B, 7A, 7B, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -3698,11 +2363,6 @@
           <t>344</t>
         </is>
       </c>
-      <c r="B274" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 2, 3A, 3B, 4, 5, 6, 7A, 7B, 7C, 7D, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -3710,11 +2370,6 @@
           <t>345</t>
         </is>
       </c>
-      <c r="B275" t="inlineStr">
-        <is>
-          <t>1, 10A, 10B1, 10B2A1A, 10B2B, 10B2C, 11, 12, 13, 2, 3A, 3B, 3C, 4, 5, 6, 7, 8, 9A, 9B, 9C, 9D, 9E, 9F, 9G</t>
-        </is>
-      </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -3722,11 +2377,6 @@
           <t>346</t>
         </is>
       </c>
-      <c r="B276" t="inlineStr">
-        <is>
-          <t>10A1, 10A2, 10B, 11, 12, 13, 14, 15, 16, 17, 18, 19, 1A1A, 1A1B, 1A1C, 1A1D, 1A1E, 1A1F, 1A1G, 1A1H, 1A1I, 20, 21, 22, 23, 24, 25, 26, 27, 29, 2A, 2B, 3A, 3B, 4, 5A, 5B, 6, 7, 8, 9A, 9B</t>
-        </is>
-      </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -3734,11 +2384,6 @@
           <t>347</t>
         </is>
       </c>
-      <c r="B277" t="inlineStr">
-        <is>
-          <t>10A1A1A1A, 10B, 11A, 11B, 12A, 12B, 13, 14, 15, 16, 17, 18, 19, 1A, 1B1A, 1B1B, 1B2, 1B3, 2, 20, 21, 22, 23, 24, 3A, 3B, 4A1, 4A2, 4A3, 4B1, 4B2, 5A1, 5A2, 5B, 6A1, 6A2, 6B, 7A, 7B, 8A1, 8A2, 8B, 9</t>
-        </is>
-      </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -3746,11 +2391,6 @@
           <t>348</t>
         </is>
       </c>
-      <c r="B278" t="inlineStr">
-        <is>
-          <t>10, 11, 12, 13A, 13B, 14A, 14B, 15, 16A, 16B, 16C, 16D, 17, 18, 19A, 19B, 1A, 1B, 1C, 1D, 1E, 2, 20, 21, 22A, 22B, 23A, 23B, 23C, 24, 25A, 25B, 25C, 26A, 26B, 26C, 27, 28, 29A, 29B, 3, 4, 5, 6, 7, 8, 9A, 9B, 9C, 9D, 9E, 9F</t>
-        </is>
-      </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -3758,11 +2398,6 @@
           <t>349</t>
         </is>
       </c>
-      <c r="B279" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -3770,11 +2405,6 @@
           <t>35</t>
         </is>
       </c>
-      <c r="B280" t="inlineStr">
-        <is>
-          <t>10, 11, 12, 13, 14, 1A, 1B, 2, 3, 4, 5, 6, 7A1, 7A2, 7B, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -3782,11 +2412,6 @@
           <t>350</t>
         </is>
       </c>
-      <c r="B281" t="inlineStr">
-        <is>
-          <t>10A, 10B, 11A, 11B, 11C, 12A, 12B, 13A1, 13A2, 13A3, 13B, 14, 15, 16A, 16B, 16C, 17, 18, 19A, 19B, 1A1, 1A2, 1A3A, 1A3B, 1B, 2, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
@@ -3794,11 +2419,6 @@
           <t>351</t>
         </is>
       </c>
-      <c r="B282" t="inlineStr">
-        <is>
-          <t>10, 11, 12, 13, 14, 15, 16, 17, 1A1A1A1, 2, 3A, 3B, 4, 5, 6, 7A, 7B, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -3806,11 +2426,6 @@
           <t>352</t>
         </is>
       </c>
-      <c r="B283" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -3818,11 +2433,6 @@
           <t>353</t>
         </is>
       </c>
-      <c r="B284" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 2C, 2D, 2E, 2F, 2G, 2H, 2I, 2J, 2K, 2L, 2M, 3, 4A, 4B, 4C</t>
-        </is>
-      </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
@@ -3830,11 +2440,6 @@
           <t>354</t>
         </is>
       </c>
-      <c r="B285" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 23, 24, 25, 26, 27, 3A, 3B, 3C, 4, 5, 6, 7A, 7B, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
@@ -3842,11 +2447,6 @@
           <t>355</t>
         </is>
       </c>
-      <c r="B286" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 2A1, 2A2, 2B, 3, 4, 5A, 5B1, 5B2, 6A, 6B, 6C1, 6C2, 7A, 7B, 7C1, 7C2, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
@@ -3854,11 +2454,6 @@
           <t>356</t>
         </is>
       </c>
-      <c r="B287" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 2A, 2B, 3, 4A, 4B, 5A, 5B, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
@@ -3866,11 +2461,6 @@
           <t>357</t>
         </is>
       </c>
-      <c r="B288" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12A, 12B, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 23A, 23B, 23C, 24, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
@@ -3878,11 +2468,6 @@
           <t>358</t>
         </is>
       </c>
-      <c r="B289" t="inlineStr">
-        <is>
-          <t>1, 2, 3</t>
-        </is>
-      </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
@@ -3890,11 +2475,6 @@
           <t>36</t>
         </is>
       </c>
-      <c r="B290" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12A, 12B, 12C, 12D, 12E, 13A, 13B, 14, 15, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
@@ -3902,11 +2482,6 @@
           <t>37</t>
         </is>
       </c>
-      <c r="B291" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 2, 3, 4, 5, 6, 7A, 7B, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
@@ -3914,11 +2489,6 @@
           <t>38</t>
         </is>
       </c>
-      <c r="B292" t="inlineStr">
-        <is>
-          <t>1, 10, 11A, 11B, 11C, 12A1, 12A2, 12B1, 12B2, 13, 14, 2A1, 2A2, 2B, 2C, 3A, 3B, 4, 5A, 5B, 6, 7, 8A, 8B, 9A, 9B</t>
-        </is>
-      </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
@@ -3926,11 +2496,6 @@
           <t>39</t>
         </is>
       </c>
-      <c r="B293" t="inlineStr">
-        <is>
-          <t>10, 11, 1A, 1B, 2, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -3938,11 +2503,6 @@
           <t>4</t>
         </is>
       </c>
-      <c r="B294" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6, 7, 8</t>
-        </is>
-      </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -3950,11 +2510,6 @@
           <t>40</t>
         </is>
       </c>
-      <c r="B295" t="inlineStr">
-        <is>
-          <t>1A, 1B, 1C, 1D, 1E, 2A, 2B, 2C, 3, 4</t>
-        </is>
-      </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
@@ -3962,11 +2517,6 @@
           <t>41</t>
         </is>
       </c>
-      <c r="B296" t="inlineStr">
-        <is>
-          <t>1A, 1B, 1C, 1D, 2, 3A, 3B, 3C, 3D, 3E, 3F1A, 3F1B, 3F2, 3G1, 3G2, 3H1A, 3H1B, 3H2, 3I1, 3I2, 3J1A, 3J1B, 3J2, 3K1, 3K2, 3L, 3M1, 3M2, 3N1A, 3N2, 3N3, 3N4</t>
-        </is>
-      </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
@@ -3974,11 +2524,6 @@
           <t>42</t>
         </is>
       </c>
-      <c r="B297" t="inlineStr">
-        <is>
-          <t>1A1, 1A2, 1A3, 1B, 1C, 2, 3A, 3B1, 3B2, 3C, 3D, 3E, 3F, 3G, 4, 5, 6A, 6B</t>
-        </is>
-      </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
@@ -3986,11 +2531,6 @@
           <t>43</t>
         </is>
       </c>
-      <c r="B298" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 3, 4, 5, 6, 7</t>
-        </is>
-      </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
@@ -3998,11 +2538,6 @@
           <t>44</t>
         </is>
       </c>
-      <c r="B299" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 2A, 2B, 2C, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
@@ -4010,11 +2545,6 @@
           <t>45</t>
         </is>
       </c>
-      <c r="B300" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -4022,11 +2552,6 @@
           <t>46</t>
         </is>
       </c>
-      <c r="B301" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 2, 3, 4, 5A1, 5A2, 5B, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
@@ -4034,11 +2559,6 @@
           <t>47</t>
         </is>
       </c>
-      <c r="B302" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 2, 3, 4, 5A, 5B, 5C, 5D, 5E, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
@@ -4046,11 +2566,6 @@
           <t>48</t>
         </is>
       </c>
-      <c r="B303" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 3, 4, 5, 6</t>
-        </is>
-      </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
@@ -4058,11 +2573,6 @@
           <t>49</t>
         </is>
       </c>
-      <c r="B304" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 2, 3, 4, 5, 6, 7, 8A, 8B, 9</t>
-        </is>
-      </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
@@ -4070,11 +2580,6 @@
           <t>5</t>
         </is>
       </c>
-      <c r="B305" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
-      </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
@@ -4082,11 +2587,6 @@
           <t>50</t>
         </is>
       </c>
-      <c r="B306" t="inlineStr">
-        <is>
-          <t>1A1, 1B, 1C, 2, 3, 4A1, 4A2A1, 4A2B, 4A2C, 4A2D, 4A2E, 4B</t>
-        </is>
-      </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -4094,11 +2594,6 @@
           <t>51</t>
         </is>
       </c>
-      <c r="B307" t="inlineStr">
-        <is>
-          <t>1A, 1B1, 1B2, 1B3, 2, 3, 4, 5</t>
-        </is>
-      </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
@@ -4106,11 +2601,6 @@
           <t>52</t>
         </is>
       </c>
-      <c r="B308" t="inlineStr">
-        <is>
-          <t>10, 11A, 11B, 1A, 1B, 2, 3, 4, 5A, 5B, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
@@ -4118,11 +2608,6 @@
           <t>53</t>
         </is>
       </c>
-      <c r="B309" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
@@ -4130,11 +2615,6 @@
           <t>54</t>
         </is>
       </c>
-      <c r="B310" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
@@ -4142,11 +2622,6 @@
           <t>55</t>
         </is>
       </c>
-      <c r="B311" t="inlineStr">
-        <is>
-          <t>1, 2, 3</t>
-        </is>
-      </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
@@ -4154,11 +2629,6 @@
           <t>56</t>
         </is>
       </c>
-      <c r="B312" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4A, 4B, 4C, 4D1, 4D2, 5, 6</t>
-        </is>
-      </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
@@ -4166,11 +2636,6 @@
           <t>57</t>
         </is>
       </c>
-      <c r="B313" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6, 7</t>
-        </is>
-      </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
@@ -4178,11 +2643,6 @@
           <t>58</t>
         </is>
       </c>
-      <c r="B314" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 2, 3A, 3B, 4A, 4B, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
@@ -4190,11 +2650,6 @@
           <t>59</t>
         </is>
       </c>
-      <c r="B315" t="inlineStr">
-        <is>
-          <t>10A, 10B, 11, 12, 13, 14, 15, 16, 17, 1A, 1B, 2A, 2B, 3, 4, 5, 6A, 6B, 7, 8, 9A, 9B</t>
-        </is>
-      </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
@@ -4202,11 +2657,6 @@
           <t>6</t>
         </is>
       </c>
-      <c r="B316" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2, 3, 4A, 4B, 5A, 5B, 6A, 6B, 7A, 7B, 8A, 8B1, 8B2, 8B3</t>
-        </is>
-      </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
@@ -4214,11 +2664,6 @@
           <t>60</t>
         </is>
       </c>
-      <c r="B317" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
@@ -4226,11 +2671,6 @@
           <t>61</t>
         </is>
       </c>
-      <c r="B318" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 2, 3, 4A, 4B, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
@@ -4238,11 +2678,6 @@
           <t>62</t>
         </is>
       </c>
-      <c r="B319" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
@@ -4250,11 +2685,6 @@
           <t>63</t>
         </is>
       </c>
-      <c r="B320" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
@@ -4262,11 +2692,6 @@
           <t>64</t>
         </is>
       </c>
-      <c r="B321" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 3, 4, 5, 6, 7</t>
-        </is>
-      </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
@@ -4274,11 +2699,6 @@
           <t>65</t>
         </is>
       </c>
-      <c r="B322" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 2, 3, 4, 5, 6A, 6B, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
@@ -4286,11 +2706,6 @@
           <t>66</t>
         </is>
       </c>
-      <c r="B323" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 2A, 2B, 3, 4, 5, 6, 7, 8A, 8B, 9</t>
-        </is>
-      </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
@@ -4298,11 +2713,6 @@
           <t>67</t>
         </is>
       </c>
-      <c r="B324" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4A1, 4A2, 4B, 5, 6, 7A, 7B, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
@@ -4310,11 +2720,6 @@
           <t>68</t>
         </is>
       </c>
-      <c r="B325" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5A, 5B, 6A, 6B, 6C, 6D, 7</t>
-        </is>
-      </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
@@ -4322,11 +2727,6 @@
           <t>69</t>
         </is>
       </c>
-      <c r="B326" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4</t>
-        </is>
-      </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
@@ -4334,11 +2734,6 @@
           <t>7</t>
         </is>
       </c>
-      <c r="B327" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
@@ -4346,11 +2741,6 @@
           <t>70</t>
         </is>
       </c>
-      <c r="B328" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 3, 4, 5</t>
-        </is>
-      </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
@@ -4358,11 +2748,6 @@
           <t>71</t>
         </is>
       </c>
-      <c r="B329" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4</t>
-        </is>
-      </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
@@ -4370,11 +2755,6 @@
           <t>72</t>
         </is>
       </c>
-      <c r="B330" t="inlineStr">
-        <is>
-          <t>1, 10, 11A, 11B, 12, 13, 14, 15, 16, 2, 3, 4, 5, 6A, 6B, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
@@ -4382,11 +2762,6 @@
           <t>73</t>
         </is>
       </c>
-      <c r="B331" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 2, 3, 4, 5A, 5B, 6, 7, 8A, 8B, 9</t>
-        </is>
-      </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
@@ -4394,11 +2769,6 @@
           <t>74</t>
         </is>
       </c>
-      <c r="B332" t="inlineStr">
-        <is>
-          <t>1A, 1B, 1C, 1D, 1E, 1F, 1G, 1H, 1I, 1J, 2A, 2B, 2C, 2D, 2E, 2F, 2G, 2H, 2I, 2J, 2K, 2L, 2M, 2N, 2O, 2P, 2Q, 2R, 2S, 2T, 2U</t>
-        </is>
-      </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
@@ -4406,11 +2776,6 @@
           <t>75</t>
         </is>
       </c>
-      <c r="B333" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
@@ -4418,11 +2783,6 @@
           <t>76</t>
         </is>
       </c>
-      <c r="B334" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2A, 2B, 2C, 2D, 2E, 2F, 2G, 2H, 2I</t>
-        </is>
-      </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
@@ -4430,11 +2790,6 @@
           <t>77</t>
         </is>
       </c>
-      <c r="B335" t="inlineStr">
-        <is>
-          <t>1, 2, 3A, 3B, 4</t>
-        </is>
-      </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
@@ -4442,11 +2797,6 @@
           <t>78</t>
         </is>
       </c>
-      <c r="B336" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
@@ -4454,11 +2804,6 @@
           <t>79</t>
         </is>
       </c>
-      <c r="B337" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
@@ -4466,11 +2811,6 @@
           <t>8</t>
         </is>
       </c>
-      <c r="B338" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15A, 15B1, 15B2, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
@@ -4478,11 +2818,6 @@
           <t>80</t>
         </is>
       </c>
-      <c r="B339" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
@@ -4490,11 +2825,6 @@
           <t>81</t>
         </is>
       </c>
-      <c r="B340" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
@@ -4502,11 +2832,6 @@
           <t>82</t>
         </is>
       </c>
-      <c r="B341" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
@@ -4514,11 +2839,6 @@
           <t>83</t>
         </is>
       </c>
-      <c r="B342" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
@@ -4526,11 +2846,6 @@
           <t>84</t>
         </is>
       </c>
-      <c r="B343" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B</t>
-        </is>
-      </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
@@ -4538,11 +2853,6 @@
           <t>85</t>
         </is>
       </c>
-      <c r="B344" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
@@ -4550,11 +2860,6 @@
           <t>86</t>
         </is>
       </c>
-      <c r="B345" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
@@ -4562,11 +2867,6 @@
           <t>87</t>
         </is>
       </c>
-      <c r="B346" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
-      </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
@@ -4574,11 +2874,6 @@
           <t>88</t>
         </is>
       </c>
-      <c r="B347" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
@@ -4586,11 +2881,6 @@
           <t>89</t>
         </is>
       </c>
-      <c r="B348" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 2, 3, 4A, 4B, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
@@ -4598,11 +2888,6 @@
           <t>9</t>
         </is>
       </c>
-      <c r="B349" t="inlineStr">
-        <is>
-          <t>1, 10, 2, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
@@ -4610,11 +2895,6 @@
           <t>90</t>
         </is>
       </c>
-      <c r="B350" t="inlineStr">
-        <is>
-          <t>10A, 10B, 11, 12, 13A, 13B, 1A, 1B, 1C, 2, 3, 4, 5A, 5B, 6, 7, 8A1, 8A2, 8B, 9A, 9B</t>
-        </is>
-      </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
@@ -4622,11 +2902,6 @@
           <t>91</t>
         </is>
       </c>
-      <c r="B351" t="inlineStr">
-        <is>
-          <t>1, 2, 3</t>
-        </is>
-      </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
@@ -4634,11 +2909,6 @@
           <t>92</t>
         </is>
       </c>
-      <c r="B352" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
@@ -4646,11 +2916,6 @@
           <t>93</t>
         </is>
       </c>
-      <c r="B353" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 3, 30, 31, 32, 33, 34, 35, 36, 37, 38A, 38B, 38C, 39, 4, 40, 41, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
@@ -4658,11 +2923,6 @@
           <t>94</t>
         </is>
       </c>
-      <c r="B354" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6, 7</t>
-        </is>
-      </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
@@ -4670,11 +2930,6 @@
           <t>95</t>
         </is>
       </c>
-      <c r="B355" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
@@ -4682,11 +2937,6 @@
           <t>96</t>
         </is>
       </c>
-      <c r="B356" t="inlineStr">
-        <is>
-          <t>10, 11, 12, 13A, 13B, 14, 15, 16, 17, 18, 19, 1A, 1B, 2, 20, 21A, 21B, 22A, 22B, 22C, 3, 4A, 4B, 4C, 5, 6A, 6B, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
@@ -4694,11 +2944,6 @@
           <t>97</t>
         </is>
       </c>
-      <c r="B357" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 2C, 3, 4, 5</t>
-        </is>
-      </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
@@ -4706,21 +2951,11 @@
           <t>98</t>
         </is>
       </c>
-      <c r="B358" t="inlineStr">
-        <is>
-          <t>10, 1A, 1B, 1C, 2, 3, 4, 5, 6, 7, 8, 9A, 9B, 9C, 9D, 9E, 9F, 9G, 9H</t>
-        </is>
-      </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
           <t>99</t>
-        </is>
-      </c>
-      <c r="B359" t="inlineStr">
-        <is>
-          <t>-</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 39 village workbooks (randomwalk-TRX50-WS 2026-10-09T16:20:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Edur_13.477828_80.078782.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Edur_13.477828_80.078782.xlsx
@@ -494,6 +494,11 @@
           <t>103</t>
         </is>
       </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 2, 3, 4, 5, 6, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -501,6 +506,11 @@
           <t>104</t>
         </is>
       </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 10C, 10D, 11, 12, 13, 2, 3, 4, 5, 6, 7, 8A, 8B, 9A, 9B, 9C</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -508,6 +518,11 @@
           <t>105</t>
         </is>
       </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 12, 2A, 2B, 2C, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -515,6 +530,11 @@
           <t>106</t>
         </is>
       </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11, 12, 13, 14, 2, 3, 4, 5, 6, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -522,6 +542,11 @@
           <t>107</t>
         </is>
       </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 1A, 1B, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -529,6 +554,11 @@
           <t>108</t>
         </is>
       </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -536,6 +566,11 @@
           <t>109</t>
         </is>
       </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -543,6 +578,11 @@
           <t>11</t>
         </is>
       </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2, 3, 4, 5, 6A, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -550,6 +590,11 @@
           <t>110</t>
         </is>
       </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -557,6 +602,11 @@
           <t>111</t>
         </is>
       </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B, 6, 7, 8A, 8B</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -564,6 +614,11 @@
           <t>112</t>
         </is>
       </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A, 3B, 4, 5, 6A, 6B, 6C, 6D, 6E, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -571,6 +626,11 @@
           <t>113</t>
         </is>
       </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 1A, 1B, 1C, 1D, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -578,6 +638,11 @@
           <t>114</t>
         </is>
       </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>10, 11A, 11B, 12A, 12B, 13, 1A, 1B, 2, 3, 4, 5, 6, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -585,6 +650,11 @@
           <t>115</t>
         </is>
       </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 3C, 3D, 3E, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -592,6 +662,11 @@
           <t>116</t>
         </is>
       </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>1, 10, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -599,6 +674,11 @@
           <t>117</t>
         </is>
       </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -606,6 +686,11 @@
           <t>118</t>
         </is>
       </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -613,6 +698,11 @@
           <t>119</t>
         </is>
       </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -620,6 +710,11 @@
           <t>12</t>
         </is>
       </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -627,6 +722,11 @@
           <t>120</t>
         </is>
       </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -634,6 +734,11 @@
           <t>121</t>
         </is>
       </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2, 3A, 3B, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -641,6 +746,11 @@
           <t>122</t>
         </is>
       </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 1A, 1B, 2, 20, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -648,6 +758,11 @@
           <t>123</t>
         </is>
       </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 2A, 2B, 3, 4A, 4B, 5A, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -655,6 +770,11 @@
           <t>124</t>
         </is>
       </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 2A, 2B, 3A, 3B, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -662,6 +782,11 @@
           <t>125</t>
         </is>
       </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2, 3A, 3B, 3C, 4A, 4B, 5A, 5B, 6</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -669,6 +794,11 @@
           <t>126</t>
         </is>
       </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -676,6 +806,11 @@
           <t>127</t>
         </is>
       </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>10A, 10B, 11, 12, 13, 14A1, 14A2, 14B, 15A, 15B, 1A, 1B, 2A, 2B, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -683,6 +818,11 @@
           <t>128</t>
         </is>
       </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>10A, 10B, 11, 12A, 12B, 13, 14, 1A1, 1B, 1C, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -690,6 +830,11 @@
           <t>129</t>
         </is>
       </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13A, 13B, 13C, 13D, 14, 15, 16, 1A, 1B, 1C, 2, 3, 4, 5, 6A, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -697,6 +842,11 @@
           <t>13</t>
         </is>
       </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 1A, 1B, 2, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -704,6 +854,11 @@
           <t>130</t>
         </is>
       </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -711,6 +866,11 @@
           <t>131</t>
         </is>
       </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -718,6 +878,11 @@
           <t>132</t>
         </is>
       </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>1, 10, 2, 3, 4, 5, 6A, 6B, 6C1, 6C2, 6D1, 6D2, 6E, 6F1, 6F2, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -725,6 +890,11 @@
           <t>133</t>
         </is>
       </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 10C, 11, 12, 13, 14, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -732,6 +902,11 @@
           <t>134</t>
         </is>
       </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14A, 14B, 2, 3, 4, 5, 6, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -739,6 +914,11 @@
           <t>135</t>
         </is>
       </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -746,6 +926,11 @@
           <t>136</t>
         </is>
       </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -753,6 +938,11 @@
           <t>137</t>
         </is>
       </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 12A, 12B, 2, 3, 4A, 4B, 5A, 5B, 5C, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -760,6 +950,11 @@
           <t>138</t>
         </is>
       </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F, 1G, 1H, 1I, 2A, 2B, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -767,6 +962,11 @@
           <t>139</t>
         </is>
       </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 1A, 1B, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -774,6 +974,11 @@
           <t>14</t>
         </is>
       </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -781,6 +986,11 @@
           <t>140</t>
         </is>
       </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -788,6 +998,11 @@
           <t>141</t>
         </is>
       </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>1, 10, 2, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -795,6 +1010,11 @@
           <t>142</t>
         </is>
       </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11A, 11B, 11C, 11D, 2, 3, 4, 5, 6, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -802,6 +1022,11 @@
           <t>143</t>
         </is>
       </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -809,6 +1034,11 @@
           <t>144</t>
         </is>
       </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>1, 10, 2, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -816,6 +1046,11 @@
           <t>145</t>
         </is>
       </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13A1, 13A2, 13B, 14A, 14B, 14C, 15A, 15B, 16A, 16B, 16C, 16D, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -823,6 +1058,11 @@
           <t>146</t>
         </is>
       </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>1, 10, 2, 3, 4A, 4B, 5A, 5B, 6, 7A, 7B, 8, 9A, 9B1, 9B2</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -830,6 +1070,11 @@
           <t>147</t>
         </is>
       </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 12, 13, 14, 2A, 2B, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -837,6 +1082,11 @@
           <t>148</t>
         </is>
       </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>10A, 10B, 1A, 1B, 2A1, 2A2, 2B, 3, 4, 5, 6, 7A, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -844,6 +1094,11 @@
           <t>149</t>
         </is>
       </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 19A, 19B, 1A, 1B, 1C, 1D, 2, 20, 21A, 21B, 22, 23A, 23B, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -851,6 +1106,11 @@
           <t>15</t>
         </is>
       </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -858,6 +1118,11 @@
           <t>150</t>
         </is>
       </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 12A, 12B, 13, 2, 3, 4, 5, 6, 7, 8A, 8B, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -865,6 +1130,11 @@
           <t>151</t>
         </is>
       </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -872,6 +1142,11 @@
           <t>152</t>
         </is>
       </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -879,6 +1154,11 @@
           <t>153</t>
         </is>
       </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B, 5C, 5D1, 5D2, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -886,6 +1166,11 @@
           <t>154</t>
         </is>
       </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 3C</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -893,6 +1178,11 @@
           <t>155</t>
         </is>
       </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -900,6 +1190,11 @@
           <t>156</t>
         </is>
       </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>1, 10, 2, 3, 4, 5, 6, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -907,6 +1202,11 @@
           <t>157</t>
         </is>
       </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -914,6 +1214,11 @@
           <t>158</t>
         </is>
       </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -921,6 +1226,11 @@
           <t>159</t>
         </is>
       </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 1A1, 1A2, 1A3, 1A4, 1B, 1C, 2A, 2B, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -928,6 +1238,11 @@
           <t>16</t>
         </is>
       </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -935,6 +1250,11 @@
           <t>160</t>
         </is>
       </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>10, 11, 1A, 1B, 2, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -942,6 +1262,11 @@
           <t>161</t>
         </is>
       </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -949,6 +1274,11 @@
           <t>162</t>
         </is>
       </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A, 12B, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 23, 24, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -956,6 +1286,11 @@
           <t>163</t>
         </is>
       </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B, 5C1, 5C2</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -963,6 +1298,11 @@
           <t>164</t>
         </is>
       </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -970,6 +1310,11 @@
           <t>165</t>
         </is>
       </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -977,6 +1322,11 @@
           <t>166</t>
         </is>
       </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2A, 2B, 3, 4A, 4B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -984,6 +1334,11 @@
           <t>167</t>
         </is>
       </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -991,6 +1346,11 @@
           <t>168</t>
         </is>
       </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -998,6 +1358,11 @@
           <t>169</t>
         </is>
       </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -1005,6 +1370,11 @@
           <t>17</t>
         </is>
       </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -1012,6 +1382,11 @@
           <t>170</t>
         </is>
       </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -1019,6 +1394,11 @@
           <t>171</t>
         </is>
       </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -1026,6 +1406,11 @@
           <t>172</t>
         </is>
       </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -1033,6 +1418,11 @@
           <t>173</t>
         </is>
       </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -1040,6 +1430,11 @@
           <t>174</t>
         </is>
       </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B, 5C, 5D, 5E, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -1047,6 +1442,11 @@
           <t>175</t>
         </is>
       </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -1054,6 +1454,11 @@
           <t>176</t>
         </is>
       </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -1061,6 +1466,11 @@
           <t>177</t>
         </is>
       </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -1068,6 +1478,11 @@
           <t>178</t>
         </is>
       </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -1075,6 +1490,11 @@
           <t>179</t>
         </is>
       </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 23, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -1082,6 +1502,11 @@
           <t>18</t>
         </is>
       </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 2, 3, 4A, 4B, 5A, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -1089,6 +1514,11 @@
           <t>180</t>
         </is>
       </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 23, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -1096,6 +1526,11 @@
           <t>181</t>
         </is>
       </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 1A, 1B, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -1103,6 +1538,11 @@
           <t>182</t>
         </is>
       </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 2, 3, 4, 5A, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -1110,11 +1550,21 @@
           <t>183</t>
         </is>
       </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 10C, 10D, 2A, 2B, 3, 4, 5, 6, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
           <t>184</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14A, 14B1, 14B2, 14B3, 15, 16, 17, 18, 2, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 39 village workbooks (randomwalk-TRX50-WS 2026-10-09T16:30:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Edur_13.477828_80.078782.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Edur_13.477828_80.078782.xlsx
@@ -1574,6 +1574,11 @@
           <t>185</t>
         </is>
       </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -1581,6 +1586,11 @@
           <t>186</t>
         </is>
       </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 23, 24, 25, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -1588,6 +1598,11 @@
           <t>187</t>
         </is>
       </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 3, 4, 5, 6, 7A1, 7A2, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -1595,6 +1610,11 @@
           <t>188</t>
         </is>
       </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -1602,6 +1622,11 @@
           <t>189</t>
         </is>
       </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 2, 3, 4, 5, 6, 7A, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -1609,6 +1634,11 @@
           <t>19</t>
         </is>
       </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>1, 10, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -1616,6 +1646,11 @@
           <t>190</t>
         </is>
       </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -1623,6 +1658,11 @@
           <t>191</t>
         </is>
       </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 2A, 2B, 2C1, 2C2, 3, 4, 5, 6, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -1630,6 +1670,11 @@
           <t>192</t>
         </is>
       </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -1637,6 +1682,11 @@
           <t>193</t>
         </is>
       </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -1644,6 +1694,11 @@
           <t>194</t>
         </is>
       </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>10, 11, 1A, 1B, 2, 3, 4, 5, 6A, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -1651,6 +1706,11 @@
           <t>195</t>
         </is>
       </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 2, 3, 4, 5, 6A, 6B, 6C, 6D, 6E, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -1658,6 +1718,11 @@
           <t>196</t>
         </is>
       </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 1A, 1B, 1C, 2A, 2B, 3A, 3B, 3C, 3D, 3E, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -1665,6 +1730,11 @@
           <t>197</t>
         </is>
       </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 12, 13, 14, 15, 16, 17, 18, 19, 2, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -1672,6 +1742,11 @@
           <t>198</t>
         </is>
       </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A, 12B, 12C, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -1679,6 +1754,11 @@
           <t>199</t>
         </is>
       </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 2, 3, 4, 5, 6A, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -1686,6 +1766,11 @@
           <t>2</t>
         </is>
       </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -1693,6 +1778,11 @@
           <t>20</t>
         </is>
       </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 2, 3, 4, 5, 6, 7A, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -1700,6 +1790,11 @@
           <t>200</t>
         </is>
       </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 3, 4, 5, 6, 7A, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -1707,6 +1802,11 @@
           <t>201</t>
         </is>
       </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -1714,6 +1814,11 @@
           <t>202</t>
         </is>
       </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 23, 24, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -1721,6 +1826,11 @@
           <t>203</t>
         </is>
       </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -1728,6 +1838,11 @@
           <t>204</t>
         </is>
       </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19A, 19B, 2, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 3, 30, 31, 32A, 32B, 33, 34, 35, 36, 37A, 37B, 37C, 38, 39, 40, 41, 42A, 42B, 43, 4A, 4B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -1735,6 +1850,11 @@
           <t>205</t>
         </is>
       </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18A, 18B, 19, 2, 20, 21, 22, 23A, 23B, 24, 25, 26, 27, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -1742,6 +1862,11 @@
           <t>206</t>
         </is>
       </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 3, 4, 5, 6, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -1749,6 +1874,11 @@
           <t>207</t>
         </is>
       </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11, 12, 13, 14, 15, 16, 17, 18, 19A, 19B, 2, 20, 21, 3, 4A, 4B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -1756,6 +1886,11 @@
           <t>208</t>
         </is>
       </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 2, 3A1A, 3A1B, 3A2A, 3A2B, 3B, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -1763,11 +1898,21 @@
           <t>209</t>
         </is>
       </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 2, 3, 4, 5A1, 5A2, 5B, 6, 7A, 7B1, 7B2, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
           <t>21</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 2, 3, 4, 5A, 5B, 6, 7, 8, 9</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 39 village workbooks (randomwalk-TRX50-WS 2026-10-09T18:20:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Edur_13.477828_80.078782.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Edur_13.477828_80.078782.xlsx
@@ -1922,6 +1922,11 @@
           <t>210</t>
         </is>
       </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16A, 16B, 16C, 17, 18, 19, 2, 20A, 20B, 21, 22, 23, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -1929,6 +1934,11 @@
           <t>211</t>
         </is>
       </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -1936,6 +1946,11 @@
           <t>212</t>
         </is>
       </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>10, 11, 12A, 12B, 13, 1A, 1B, 2A, 2B, 3, 4, 5, 6A, 6B, 6C, 7A, 7B, 7C, 8, 9A, 9B, 9C</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -1943,6 +1958,11 @@
           <t>213</t>
         </is>
       </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -1950,6 +1970,11 @@
           <t>214</t>
         </is>
       </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>11, 12, 13, 14, 15, 16, 17, 18, 19, 1A, 2, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 3, 30, 31, 32, 33, 34, 35, 36, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -1957,11 +1982,21 @@
           <t>215</t>
         </is>
       </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14A1A1, 14A2, 14B, 14C, 14D, 14E, 14F1A, 14F2, 15, 16, 17, 18, 19A, 19B, 2, 20, 21, 22, 23, 3, 4A1A, 4A1B, 4A1C, 4A2, 4A3, 4A4, 4A5, 4B, 4C, 4D, 5, 6, 7A, 7B, 7C, 7D, 7E, 8, 9A1, 9A2, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
           <t>216</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>1, 10, 2, 3, 4A, 4B, 5, 6, 7, 8A1A1A, 8A1B, 8A1C, 8A2, 8B, 9</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 40 village workbooks (randomwalk-TRX50-WS 2026-10-09T18:30:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Edur_13.477828_80.078782.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Edur_13.477828_80.078782.xlsx
@@ -2006,6 +2006,11 @@
           <t>217</t>
         </is>
       </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 11C, 12A, 12B, 2A, 2B, 2C, 2D, 2E, 2F, 3, 4A, 4B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -2013,6 +2018,11 @@
           <t>218</t>
         </is>
       </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B1, 2B2</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -2020,6 +2030,11 @@
           <t>219</t>
         </is>
       </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7A1, 7A2, 7B, 7C, 7D, 7E, 7F, 7G, 8</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -2027,6 +2042,11 @@
           <t>22</t>
         </is>
       </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>1, 10, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -2034,6 +2054,11 @@
           <t>220</t>
         </is>
       </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13A, 13B, 14, 15, 16, 17A, 17B, 17C, 17D, 18A, 18B, 19A, 19B, 2, 20, 21, 22A1, 22A2, 22B, 23, 24, 25, 26, 27A, 27B, 27C, 28A, 28B, 28C, 3A, 3B, 3C1, 3C2, 3D1, 3D2A, 3D2B, 3E, 3F, 4A, 4B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -2041,6 +2066,11 @@
           <t>221</t>
         </is>
       </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 23, 3, 4, 5, 6, 7A, 7B, 7C, 7D, 7E, 7F, 7G, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -2048,6 +2078,11 @@
           <t>222</t>
         </is>
       </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>10, 11, 12A, 12B, 13A, 13B, 14A, 14B, 15, 16, 17A, 17B, 18, 19, 1A, 1B, 2, 20, 21, 22, 3, 4, 5A, 5B, 6A, 6B, 7A, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -2055,6 +2090,11 @@
           <t>223</t>
         </is>
       </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 10C, 10D, 11A, 11B, 12, 13A, 13B, 13C, 13D, 13E, 13F, 14A, 14B, 15A, 15B, 16A, 16B, 2A, 2B, 3A1, 3A2, 3B, 4A, 4B, 5, 6A, 6B, 7, 8, 9A, 9B, 9C, 9D</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -2062,6 +2102,11 @@
           <t>224</t>
         </is>
       </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>1, 10A1A1A1A, 10A1B, 10A1C, 10A1D, 10A1E, 10A2, 10A3, 10B, 11, 12, 13A, 13B, 14, 15, 16, 17, 18, 2, 3A, 3B, 4, 5, 6, 7A, 7B, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -2069,6 +2114,11 @@
           <t>225</t>
         </is>
       </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A1A1, 12A1B, 12A2, 12B, 13A, 13B, 13C, 13D, 13E, 14A1A, 14A1B, 14A2, 14B, 14C1, 14C2, 14C3, 15A1A, 15A2, 15B, 16A1A, 16A1B, 16A2, 16B, 17, 18, 2A1, 2A2, 2B, 3, 4A, 4B, 4C, 4D, 5A, 5B, 6A, 6B, 6C1, 6C2, 6D, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -2076,6 +2126,11 @@
           <t>226</t>
         </is>
       </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2A, 2B1A, 2B1B, 2B2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -2083,6 +2138,11 @@
           <t>227</t>
         </is>
       </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -2090,6 +2150,11 @@
           <t>228</t>
         </is>
       </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F, 1G, 1H, 1I, 1J, 1K, 2, 3, 4, 5, 6A, 6B, 7</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -2097,6 +2162,11 @@
           <t>229</t>
         </is>
       </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -2104,6 +2174,11 @@
           <t>23</t>
         </is>
       </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8A, 8B</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -2111,6 +2186,11 @@
           <t>230</t>
         </is>
       </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -2118,6 +2198,11 @@
           <t>231</t>
         </is>
       </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 1A, 1B, 2, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -2125,6 +2210,11 @@
           <t>232</t>
         </is>
       </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -2132,6 +2222,11 @@
           <t>233</t>
         </is>
       </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A, 12B, 13A, 13B, 13C, 14, 2, 3, 4, 5A, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -2139,6 +2234,11 @@
           <t>234</t>
         </is>
       </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>10, 11, 1A, 1B, 1C, 2, 3, 4, 5, 6A, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -2146,6 +2246,11 @@
           <t>235</t>
         </is>
       </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4, 5, 6, 7, 8A, 8B</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -2153,6 +2258,11 @@
           <t>236</t>
         </is>
       </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -2160,6 +2270,11 @@
           <t>237</t>
         </is>
       </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -2167,6 +2282,11 @@
           <t>238</t>
         </is>
       </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -2174,6 +2294,11 @@
           <t>239</t>
         </is>
       </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 2C, 3A, 3B, 3C, 3D, 3E, 3F, 3G, 3H, 3I, 3J, 3K, 3L, 3M, 3N, 3O, 3P, 3Q, 3R, 3S, 3T, 3U, 3V, 3W, 3X, 4A, 4B, 5A, 5B, 5C, 6A, 6B, 6C, 6D, 6E, 6F, 6G, 7, 8, 9A, 9B, 9C</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -2181,6 +2306,11 @@
           <t>24</t>
         </is>
       </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>1, 10A1, 10A2, 10A3, 10B, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -2188,6 +2318,11 @@
           <t>240</t>
         </is>
       </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D, 2E, 2F, 2G, 2H, 2I, 3A, 3B, 3C, 3D, 3E, 3F, 4, 5, 6, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -2195,6 +2330,11 @@
           <t>241</t>
         </is>
       </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -2202,6 +2342,11 @@
           <t>242</t>
         </is>
       </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -2209,6 +2354,11 @@
           <t>243</t>
         </is>
       </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -2216,6 +2366,11 @@
           <t>244</t>
         </is>
       </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -2223,6 +2378,11 @@
           <t>245</t>
         </is>
       </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -2230,6 +2390,11 @@
           <t>246</t>
         </is>
       </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -2237,6 +2402,11 @@
           <t>247</t>
         </is>
       </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -2244,6 +2414,11 @@
           <t>248</t>
         </is>
       </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A1, 4A2, 4B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -2251,6 +2426,11 @@
           <t>249</t>
         </is>
       </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D, 3A, 3B, 3C, 3D, 3E, 3F, 4, 5A, 5B, 5C, 6A, 6B, 7A, 7B, 8A, 8B, 9A, 9B, 9C1, 9C2A, 9C2B</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -2258,6 +2438,11 @@
           <t>25</t>
         </is>
       </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15A, 15B, 16, 17, 18A1A, 18A1B, 18A2, 18B, 19, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -2265,6 +2450,11 @@
           <t>250</t>
         </is>
       </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11, 2, 3A, 3B, 3C, 4, 5, 6A, 6B, 6C, 7A, 7B, 8A, 8B1, 8B2, 9A, 9B, 9C</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -2272,6 +2462,11 @@
           <t>251</t>
         </is>
       </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13A, 13B, 14A1A, 14A1B, 14A2, 14B, 15A, 15B, 15C, 16A, 16B, 17A1, 17A2, 17B, 18A1, 18A2, 18B, 18C, 19, 20A, 20B, 21A, 21B, 2A, 2B, 3A, 3B, 3C, 4A, 4B, 5A1, 5A2, 5A3, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -2279,6 +2474,11 @@
           <t>252</t>
         </is>
       </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 2A, 2B, 3, 4, 5A, 5B, 6</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -2286,6 +2486,11 @@
           <t>253</t>
         </is>
       </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>10, 11A, 11B, 11C, 12, 13, 1A, 1B, 1C, 2A, 2B, 2C, 3, 4, 5, 6, 7, 8A, 8B, 8C, 8D, 9A, 9B, 9C</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -2293,6 +2498,11 @@
           <t>254</t>
         </is>
       </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 11C, 11D, 11E, 11F, 11G, 11H, 11I, 12, 13, 14A, 14B, 15A, 15B, 15C, 16A, 16B, 2A1, 2A2, 2B, 3, 4, 5A, 5B, 6A, 6B, 7A, 7B, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -2300,6 +2510,11 @@
           <t>255</t>
         </is>
       </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13A, 13B1A1, 13B1A2, 13B1A3, 13B1B, 13B2, 13C, 13D1, 13D2, 14, 15A1A, 15A1B, 15A2A, 15A2B, 15B, 16, 17A, 17B1, 17B2A, 17B2B, 18, 19, 2, 20, 21, 22, 23A, 23B, 23C, 24, 3, 4, 5A, 5B1, 5B2, 5C, 5D1A, 5D1B, 5D2, 6, 7A1, 7A2A, 7A2B, 7B, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -2307,6 +2522,11 @@
           <t>256</t>
         </is>
       </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -2314,6 +2534,11 @@
           <t>257</t>
         </is>
       </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11, 12, 2A, 2B, 2C, 2D, 2E, 2F, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -2321,6 +2546,11 @@
           <t>258</t>
         </is>
       </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -2328,6 +2558,11 @@
           <t>259</t>
         </is>
       </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 3, 4A, 4B, 4C, 5, 6, 7A, 7B</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -2335,6 +2570,11 @@
           <t>26</t>
         </is>
       </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -2342,6 +2582,11 @@
           <t>260</t>
         </is>
       </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 23A, 23B, 24, 25, 26, 27, 28, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -2349,6 +2594,11 @@
           <t>261</t>
         </is>
       </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 1A, 1B, 1C, 1D, 1E, 2, 3, 4, 5, 6A, 6B, 6C, 6D, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -2356,6 +2606,11 @@
           <t>262</t>
         </is>
       </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>10, 11A, 11B, 11C, 11D, 12, 1A, 1B, 1C, 1D, 2A, 2B, 3, 4, 5, 6, 7, 8A, 8B, 9A, 9B, 9C</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -2363,6 +2618,11 @@
           <t>263</t>
         </is>
       </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 2, 3, 4, 5, 6, 7A1, 7A2, 7B, 8A, 8B, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -2370,6 +2630,11 @@
           <t>264</t>
         </is>
       </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>10, 11, 1A, 1B, 2A, 2B, 2C1, 2C2, 3A, 3B, 4A, 4B, 5A, 5B, 5C, 5D, 5E, 5F, 5G, 6, 7A, 7B, 7C, 7D, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -2377,6 +2642,11 @@
           <t>265</t>
         </is>
       </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17, 18A, 18B, 19A, 19B, 1A, 1B, 20, 21A, 21B, 22, 23A, 23B, 24, 25, 2A, 2B, 3, 4, 5, 6A, 6B, 7A, 7B, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -2384,6 +2654,11 @@
           <t>266</t>
         </is>
       </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 2A, 2B, 3A, 3B, 4, 5A, 5B, 5C, 5D, 6A, 6B, 7, 8, 9A, 9B, 9C1, 9C2, 9C3</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -2391,6 +2666,11 @@
           <t>267</t>
         </is>
       </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>10A, 10B, 10C, 10D, 11A, 11B, 11C, 12, 13, 14, 15, 16, 17, 18, 19, 1A, 1B, 1C1, 1C2, 2, 20, 21A1, 21A2, 21B, 21C, 21D, 3, 4A, 4B, 5A, 5B, 6, 7A, 7B, 8A, 8B, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -2398,6 +2678,11 @@
           <t>268</t>
         </is>
       </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13A, 13B, 14A1, 14A2, 14B, 14C, 15, 16, 17A, 17B, 18A, 18B, 19A, 19B, 2, 20, 21, 22, 23, 24, 3, 4A, 4B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -2405,6 +2690,11 @@
           <t>269</t>
         </is>
       </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A1, 12A2, 12B1, 12B2, 13, 14, 15A1, 15A2, 15B, 16, 17, 18, 19, 20, 21A1A, 21A1B1, 21B, 22, 23, 24, 25, 26, 27, 2A, 2B, 3A, 3B, 3C, 4, 5, 6, 7, 8A1, 8A2, 8B, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -2412,11 +2702,21 @@
           <t>27</t>
         </is>
       </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
           <t>270</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A, 12B, 12C, 12D, 12E, 13A, 13B, 13C, 14A, 14B, 15A, 15B, 15C, 15D, 15E, 15F, 15G, 2, 3A, 3B, 4, 5, 6A, 6B, 6C, 6D, 7, 8, 9A, 9B, 9C, 9D</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 37 village workbooks (rw-rtx-3070 2026-10-09T22:30:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Edur_13.477828_80.078782.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Edur_13.477828_80.078782.xlsx
@@ -446,6 +446,11 @@
           <t>10</t>
         </is>
       </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A, 12B, 12C, 13, 14, 15, 16, 2A, 2B, 3, 4, 5, 6, 7, 8, 9A, 9B, 9C</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -453,6 +458,11 @@
           <t>100</t>
         </is>
       </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -460,6 +470,11 @@
           <t>101</t>
         </is>
       </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -467,6 +482,11 @@
           <t>102</t>
         </is>
       </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17A, 17B, 1A, 1B, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -474,6 +494,11 @@
           <t>103</t>
         </is>
       </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 2, 3, 4, 5, 6, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -481,6 +506,11 @@
           <t>104</t>
         </is>
       </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 10C, 10D, 11, 12, 13, 2, 3, 4, 5, 6, 7, 8A, 8B, 9A, 9B, 9C</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -488,6 +518,11 @@
           <t>105</t>
         </is>
       </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 12, 2A, 2B, 2C, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -495,6 +530,11 @@
           <t>106</t>
         </is>
       </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11, 12, 13, 14, 2, 3, 4, 5, 6, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -502,6 +542,11 @@
           <t>107</t>
         </is>
       </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 1A, 1B, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -509,6 +554,11 @@
           <t>108</t>
         </is>
       </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -516,6 +566,11 @@
           <t>109</t>
         </is>
       </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -523,6 +578,11 @@
           <t>11</t>
         </is>
       </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2, 3, 4, 5, 6A, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -530,6 +590,11 @@
           <t>110</t>
         </is>
       </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -537,6 +602,11 @@
           <t>111</t>
         </is>
       </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B, 6, 7, 8A, 8B</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -544,6 +614,11 @@
           <t>112</t>
         </is>
       </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A, 3B, 4, 5, 6A, 6B, 6C, 6D, 6E, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -551,6 +626,11 @@
           <t>113</t>
         </is>
       </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 1A, 1B, 1C, 1D, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -558,6 +638,11 @@
           <t>114</t>
         </is>
       </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>10, 11A, 11B, 12A, 12B, 13, 1A, 1B, 2, 3, 4, 5, 6, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -565,6 +650,11 @@
           <t>115</t>
         </is>
       </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 3C, 3D, 3E, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -572,6 +662,11 @@
           <t>116</t>
         </is>
       </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>1, 10, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -579,6 +674,11 @@
           <t>117</t>
         </is>
       </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -586,6 +686,11 @@
           <t>118</t>
         </is>
       </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -593,6 +698,11 @@
           <t>119</t>
         </is>
       </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -600,6 +710,11 @@
           <t>12</t>
         </is>
       </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -607,6 +722,11 @@
           <t>120</t>
         </is>
       </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -614,6 +734,11 @@
           <t>121</t>
         </is>
       </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2, 3A, 3B, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -621,6 +746,11 @@
           <t>122</t>
         </is>
       </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 1A, 1B, 2, 20, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -628,6 +758,11 @@
           <t>123</t>
         </is>
       </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 2A, 2B, 3, 4A, 4B, 5A, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -635,6 +770,11 @@
           <t>124</t>
         </is>
       </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 2A, 2B, 3A, 3B, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -642,6 +782,11 @@
           <t>125</t>
         </is>
       </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2, 3A, 3B, 3C, 4A, 4B, 5A, 5B, 6</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -649,6 +794,11 @@
           <t>126</t>
         </is>
       </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -656,6 +806,11 @@
           <t>127</t>
         </is>
       </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>10A, 10B, 11, 12, 13, 14A1, 14A2, 14B, 15A, 15B, 1A, 1B, 2A, 2B, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -663,6 +818,11 @@
           <t>128</t>
         </is>
       </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>10A, 10B, 11, 12A, 12B, 13, 14, 1A1, 1B, 1C, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -670,6 +830,11 @@
           <t>129</t>
         </is>
       </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13A, 13B, 13C, 13D, 14, 15, 16, 1A, 1B, 1C, 2, 3, 4, 5, 6A, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -677,6 +842,11 @@
           <t>13</t>
         </is>
       </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 1A, 1B, 2, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -684,6 +854,11 @@
           <t>130</t>
         </is>
       </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -691,6 +866,11 @@
           <t>131</t>
         </is>
       </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -698,6 +878,11 @@
           <t>132</t>
         </is>
       </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>1, 10, 2, 3, 4, 5, 6A, 6B, 6C1, 6C2, 6D1, 6D2, 6E, 6F1, 6F2, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -705,6 +890,11 @@
           <t>133</t>
         </is>
       </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 10C, 11, 12, 13, 14, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -712,6 +902,11 @@
           <t>134</t>
         </is>
       </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14A, 14B, 2, 3, 4, 5, 6, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -719,6 +914,11 @@
           <t>135</t>
         </is>
       </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -726,6 +926,11 @@
           <t>136</t>
         </is>
       </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -733,6 +938,11 @@
           <t>137</t>
         </is>
       </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 12A, 12B, 2, 3, 4A, 4B, 5A, 5B, 5C, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -740,6 +950,11 @@
           <t>138</t>
         </is>
       </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F, 1G, 1H, 1I, 2A, 2B, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -747,6 +962,11 @@
           <t>139</t>
         </is>
       </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 1A, 1B, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -754,6 +974,11 @@
           <t>14</t>
         </is>
       </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -761,6 +986,11 @@
           <t>140</t>
         </is>
       </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -768,6 +998,11 @@
           <t>141</t>
         </is>
       </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>1, 10, 2, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -775,6 +1010,11 @@
           <t>142</t>
         </is>
       </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11A, 11B, 11C, 11D, 2, 3, 4, 5, 6, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -782,6 +1022,11 @@
           <t>143</t>
         </is>
       </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -789,6 +1034,11 @@
           <t>144</t>
         </is>
       </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>1, 10, 2, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -796,6 +1046,11 @@
           <t>145</t>
         </is>
       </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13A1, 13A2, 13B, 14A, 14B, 14C, 15A, 15B, 16A, 16B, 16C, 16D, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -803,6 +1058,11 @@
           <t>146</t>
         </is>
       </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>1, 10, 2, 3, 4A, 4B, 5A, 5B, 6, 7A, 7B, 8, 9A, 9B1, 9B2</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -810,6 +1070,11 @@
           <t>147</t>
         </is>
       </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 12, 13, 14, 2A, 2B, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -817,6 +1082,11 @@
           <t>148</t>
         </is>
       </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>10A, 10B, 1A, 1B, 2A1, 2A2, 2B, 3, 4, 5, 6, 7A, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -824,6 +1094,11 @@
           <t>149</t>
         </is>
       </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 19A, 19B, 1A, 1B, 1C, 1D, 2, 20, 21A, 21B, 22, 23A, 23B, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -831,6 +1106,11 @@
           <t>15</t>
         </is>
       </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -838,6 +1118,11 @@
           <t>150</t>
         </is>
       </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 12A, 12B, 13, 2, 3, 4, 5, 6, 7, 8A, 8B, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -845,6 +1130,11 @@
           <t>151</t>
         </is>
       </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -852,6 +1142,11 @@
           <t>152</t>
         </is>
       </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -859,6 +1154,11 @@
           <t>153</t>
         </is>
       </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B, 5C, 5D1, 5D2, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -866,6 +1166,11 @@
           <t>154</t>
         </is>
       </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 3C</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -873,6 +1178,11 @@
           <t>155</t>
         </is>
       </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -880,6 +1190,11 @@
           <t>156</t>
         </is>
       </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>1, 10, 2, 3, 4, 5, 6, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -887,6 +1202,11 @@
           <t>157</t>
         </is>
       </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -894,6 +1214,11 @@
           <t>158</t>
         </is>
       </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -901,6 +1226,11 @@
           <t>159</t>
         </is>
       </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 1A1, 1A2, 1A3, 1A4, 1B, 1C, 2A, 2B, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -908,6 +1238,11 @@
           <t>16</t>
         </is>
       </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -915,6 +1250,11 @@
           <t>160</t>
         </is>
       </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>10, 11, 1A, 1B, 2, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -922,6 +1262,11 @@
           <t>161</t>
         </is>
       </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -929,6 +1274,11 @@
           <t>162</t>
         </is>
       </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A, 12B, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 23, 24, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -936,6 +1286,11 @@
           <t>163</t>
         </is>
       </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B, 5C1, 5C2</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -943,6 +1298,11 @@
           <t>164</t>
         </is>
       </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -950,6 +1310,11 @@
           <t>165</t>
         </is>
       </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -957,6 +1322,11 @@
           <t>166</t>
         </is>
       </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2A, 2B, 3, 4A, 4B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -964,6 +1334,11 @@
           <t>167</t>
         </is>
       </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -971,6 +1346,11 @@
           <t>168</t>
         </is>
       </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -978,6 +1358,11 @@
           <t>169</t>
         </is>
       </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -985,6 +1370,11 @@
           <t>17</t>
         </is>
       </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -992,6 +1382,11 @@
           <t>170</t>
         </is>
       </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -999,6 +1394,11 @@
           <t>171</t>
         </is>
       </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -1006,6 +1406,11 @@
           <t>172</t>
         </is>
       </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -1013,6 +1418,11 @@
           <t>173</t>
         </is>
       </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -1020,6 +1430,11 @@
           <t>174</t>
         </is>
       </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B, 5C, 5D, 5E, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -1027,6 +1442,11 @@
           <t>175</t>
         </is>
       </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -1034,6 +1454,11 @@
           <t>176</t>
         </is>
       </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -1041,6 +1466,11 @@
           <t>177</t>
         </is>
       </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -1048,6 +1478,11 @@
           <t>178</t>
         </is>
       </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -1055,6 +1490,11 @@
           <t>179</t>
         </is>
       </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 23, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -1062,6 +1502,11 @@
           <t>18</t>
         </is>
       </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 2, 3, 4A, 4B, 5A, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -1069,6 +1514,11 @@
           <t>180</t>
         </is>
       </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 23, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -1076,6 +1526,11 @@
           <t>181</t>
         </is>
       </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 1A, 1B, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -1083,11 +1538,21 @@
           <t>182</t>
         </is>
       </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 2, 3, 4, 5A, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
           <t>183</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 10C, 10D, 2A, 2B, 3, 4, 5, 6, 7, 8, 9A, 9B</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 37 village workbooks (rw-rtx-3070 2026-10-09T22:40:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Edur_13.477828_80.078782.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Edur_13.477828_80.078782.xlsx
@@ -1562,6 +1562,11 @@
           <t>184</t>
         </is>
       </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14A, 14B1, 14B2, 14B3, 15, 16, 17, 18, 2, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -1569,6 +1574,11 @@
           <t>185</t>
         </is>
       </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -1576,6 +1586,11 @@
           <t>186</t>
         </is>
       </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 23, 24, 25, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -1583,6 +1598,11 @@
           <t>187</t>
         </is>
       </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 3, 4, 5, 6, 7A1, 7A2, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -1590,6 +1610,11 @@
           <t>188</t>
         </is>
       </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -1597,6 +1622,11 @@
           <t>189</t>
         </is>
       </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 2, 3, 4, 5, 6, 7A, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -1604,6 +1634,11 @@
           <t>19</t>
         </is>
       </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>1, 10, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -1611,6 +1646,11 @@
           <t>190</t>
         </is>
       </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -1618,6 +1658,11 @@
           <t>191</t>
         </is>
       </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 2A, 2B, 2C1, 2C2, 3, 4, 5, 6, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -1625,6 +1670,11 @@
           <t>192</t>
         </is>
       </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -1632,6 +1682,11 @@
           <t>193</t>
         </is>
       </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -1639,6 +1694,11 @@
           <t>194</t>
         </is>
       </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>10, 11, 1A, 1B, 2, 3, 4, 5, 6A, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -1646,6 +1706,11 @@
           <t>195</t>
         </is>
       </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 2, 3, 4, 5, 6A, 6B, 6C, 6D, 6E, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -1653,6 +1718,11 @@
           <t>196</t>
         </is>
       </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -1660,6 +1730,11 @@
           <t>197</t>
         </is>
       </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 12, 13, 14, 15, 16, 17, 18, 19, 2, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -1667,6 +1742,11 @@
           <t>198</t>
         </is>
       </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A, 12B, 12C, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -1674,6 +1754,11 @@
           <t>199</t>
         </is>
       </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 2, 3, 4, 5, 6A, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -1681,6 +1766,11 @@
           <t>2</t>
         </is>
       </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -1688,6 +1778,11 @@
           <t>20</t>
         </is>
       </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 2, 3, 4, 5, 6, 7A, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -1695,6 +1790,11 @@
           <t>200</t>
         </is>
       </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 3, 4, 5, 6, 7A, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -1702,6 +1802,11 @@
           <t>201</t>
         </is>
       </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -1709,6 +1814,11 @@
           <t>202</t>
         </is>
       </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 23, 24, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -1716,6 +1826,11 @@
           <t>203</t>
         </is>
       </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -1723,6 +1838,11 @@
           <t>204</t>
         </is>
       </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19A, 19B, 2, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 3, 30, 31, 32A, 32B, 33, 34, 35, 36, 37A, 37B, 37C, 38, 39, 40, 41, 42A, 42B, 43, 4A, 4B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -1730,6 +1850,11 @@
           <t>205</t>
         </is>
       </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18A, 18B, 19, 2, 20, 21, 22, 23A, 23B, 24, 25, 26, 27, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -1737,6 +1862,11 @@
           <t>206</t>
         </is>
       </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 3, 4, 5, 6, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -1744,6 +1874,11 @@
           <t>207</t>
         </is>
       </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11, 12, 13, 14, 15, 16, 17, 18, 19A, 19B, 2, 20, 21, 3, 4A, 4B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -1751,6 +1886,11 @@
           <t>208</t>
         </is>
       </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 2, 3A1A, 3A1B, 3A2A, 3A2B, 3B, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -1758,6 +1898,11 @@
           <t>209</t>
         </is>
       </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 2, 3, 4, 5A1, 5A2, 5B, 6, 7A, 7B1, 7B2, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -1765,6 +1910,11 @@
           <t>21</t>
         </is>
       </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 2, 3, 4, 5A, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -1772,6 +1922,11 @@
           <t>210</t>
         </is>
       </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16A, 16B, 16C, 17, 18, 19, 2, 20A, 20B, 21, 22, 23, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -1779,6 +1934,11 @@
           <t>211</t>
         </is>
       </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -1786,6 +1946,11 @@
           <t>212</t>
         </is>
       </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>10, 11, 12A, 12B, 13, 1A, 1B, 2A, 2B, 3, 4, 5, 6A, 6B, 6C, 7A, 7B, 7C, 8, 9A, 9B, 9C</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -1793,6 +1958,11 @@
           <t>213</t>
         </is>
       </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -1800,6 +1970,11 @@
           <t>214</t>
         </is>
       </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>11, 12, 13, 14, 15, 16, 17, 18, 19, 1A, 2, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 3, 30, 31, 32, 33, 34, 35, 36, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -1807,6 +1982,11 @@
           <t>215</t>
         </is>
       </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14A1A1, 14A2, 14B, 14C, 14D, 14E, 14F1A, 14F2, 15, 16, 17, 18, 19A, 19B, 2, 20, 21, 22, 23, 3, 4A1A, 4A1B, 4A1C, 4A2, 4A3, 4A4, 4A5, 4B, 4C, 4D, 5, 6, 7A, 7B, 7C, 7D, 7E, 8, 9A1, 9A2, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -1814,6 +1994,11 @@
           <t>216</t>
         </is>
       </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>1, 10, 2, 3, 4A, 4B, 5, 6, 7, 8A1A1A, 8A1B, 8A1C, 8A2, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -1821,6 +2006,11 @@
           <t>217</t>
         </is>
       </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 11C, 12A, 12B, 2A, 2B, 2C, 2D, 2E, 2F, 3, 4A, 4B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -1828,6 +2018,11 @@
           <t>218</t>
         </is>
       </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B1, 2B2</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -1835,6 +2030,11 @@
           <t>219</t>
         </is>
       </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7A1, 7A2, 7B, 7C, 7D, 7E, 7F, 7G, 8</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -1842,6 +2042,11 @@
           <t>22</t>
         </is>
       </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>1, 10, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -1849,6 +2054,11 @@
           <t>220</t>
         </is>
       </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13A, 13B, 14, 15, 16, 17A, 17B, 17C, 17D, 18A, 18B, 19A, 19B, 2, 20, 21, 22A1, 22A2, 22B, 23, 24, 25, 26, 27A, 27B, 27C, 28A, 28B, 28C, 3A, 3B, 3C1, 3C2, 3D1, 3D2A, 3D2B, 3E, 3F, 4A, 4B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -1856,6 +2066,11 @@
           <t>221</t>
         </is>
       </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 23, 3, 4, 5, 6, 7A, 7B, 7C, 7D, 7E, 7F, 7G, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -1863,6 +2078,11 @@
           <t>222</t>
         </is>
       </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>10, 11, 12A, 12B, 13A, 13B, 14A, 14B, 15, 16, 17A, 17B, 18, 19, 1A, 1B, 2, 20, 21, 22, 3, 4, 5A, 5B, 6A, 6B, 7A, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -1870,6 +2090,11 @@
           <t>223</t>
         </is>
       </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 10C, 10D, 11A, 11B, 12, 13A, 13B, 13C, 13D, 13E, 13F, 14A, 14B, 15A, 15B, 16A, 16B, 2A, 2B, 3A1, 3A2, 3B, 4A, 4B, 5, 6A, 6B, 7, 8, 9A, 9B, 9C, 9D</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -1877,6 +2102,11 @@
           <t>224</t>
         </is>
       </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>1, 10A1A1A1A, 10A1B, 10A1C, 10A1D, 10A1E, 10A2, 10A3, 10B, 11, 12, 13A, 13B, 14, 15, 16, 17, 18, 2, 3A, 3B, 4, 5, 6, 7A, 7B, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -1884,6 +2114,11 @@
           <t>225</t>
         </is>
       </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A1A1, 12A1B, 12A2, 12B, 13A, 13B, 13C, 13D, 13E, 14A1A, 14A1B, 14A2, 14B, 14C1, 14C2, 14C3, 15A1A, 15A2, 15B, 16A1A, 16A1B, 16A2, 16B, 17, 18, 2A1, 2A2, 2B, 3, 4A, 4B, 4C, 4D, 5A, 5B, 6A, 6B, 6C1, 6C2, 6D, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -1891,6 +2126,11 @@
           <t>226</t>
         </is>
       </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2A, 2B1A, 2B1B, 2B2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -1898,6 +2138,11 @@
           <t>227</t>
         </is>
       </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -1905,6 +2150,11 @@
           <t>228</t>
         </is>
       </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F, 1G, 1H, 1I, 1J, 1K, 2, 3, 4, 5, 6A, 6B, 7</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -1912,6 +2162,11 @@
           <t>229</t>
         </is>
       </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -1919,11 +2174,21 @@
           <t>23</t>
         </is>
       </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8A, 8B</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
           <t>230</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2, 3, 4, 5, 6, 7, 8, 9</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 38 village workbooks (rw-rtx-3070 2026-10-09T22:50:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Edur_13.477828_80.078782.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Edur_13.477828_80.078782.xlsx
@@ -2198,6 +2198,11 @@
           <t>231</t>
         </is>
       </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 1A, 1B, 2, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -2205,6 +2210,11 @@
           <t>232</t>
         </is>
       </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -2212,6 +2222,11 @@
           <t>233</t>
         </is>
       </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A, 12B, 13A, 13B, 13C, 14, 2, 3, 4, 5A, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -2219,6 +2234,11 @@
           <t>234</t>
         </is>
       </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>10, 11, 1A, 1B, 1C, 2, 3, 4, 5, 6A, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -2226,6 +2246,11 @@
           <t>235</t>
         </is>
       </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4, 5, 6, 7, 8A, 8B</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -2233,6 +2258,11 @@
           <t>236</t>
         </is>
       </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -2240,6 +2270,11 @@
           <t>237</t>
         </is>
       </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -2247,6 +2282,11 @@
           <t>238</t>
         </is>
       </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -2254,6 +2294,11 @@
           <t>239</t>
         </is>
       </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 2C, 3A, 3B, 3C, 3D, 3E, 3F, 3G, 3H, 3I, 3J, 3K, 3L, 3M, 3N, 3O, 3P, 3Q, 3R, 3S, 3T, 3U, 3V, 3W, 3X, 4A, 4B, 5A, 5B, 5C, 6A, 6B, 6C, 6D, 6E, 6F, 6G, 7, 8, 9A, 9B, 9C</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -2261,6 +2306,11 @@
           <t>24</t>
         </is>
       </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>1, 10A1, 10A2, 10A3, 10B, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -2268,6 +2318,11 @@
           <t>240</t>
         </is>
       </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D, 2E, 2F, 2G, 2H, 2I, 3A, 3B, 3C, 3D, 3E, 3F, 4, 5, 6, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -2275,6 +2330,11 @@
           <t>241</t>
         </is>
       </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -2282,6 +2342,11 @@
           <t>242</t>
         </is>
       </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -2289,6 +2354,11 @@
           <t>243</t>
         </is>
       </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -2296,6 +2366,11 @@
           <t>244</t>
         </is>
       </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -2303,6 +2378,11 @@
           <t>245</t>
         </is>
       </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -2310,6 +2390,11 @@
           <t>246</t>
         </is>
       </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -2317,6 +2402,11 @@
           <t>247</t>
         </is>
       </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -2324,6 +2414,11 @@
           <t>248</t>
         </is>
       </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A1, 4A2, 4B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -2331,6 +2426,11 @@
           <t>249</t>
         </is>
       </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D, 3A, 3B, 3C, 3D, 3E, 3F, 4, 5A, 5B, 5C, 6A, 6B, 7A, 7B, 8A, 8B, 9A, 9B, 9C1, 9C2A, 9C2B</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -2338,6 +2438,11 @@
           <t>25</t>
         </is>
       </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15A, 15B, 16, 17, 18A1A, 18A1B, 18A2, 18B, 19, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -2345,6 +2450,11 @@
           <t>250</t>
         </is>
       </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11, 2, 3A, 3B, 3C, 4, 5, 6A, 6B, 6C, 7A, 7B, 8A, 8B1, 8B2, 9A, 9B, 9C</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -2352,6 +2462,11 @@
           <t>251</t>
         </is>
       </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13A, 13B, 14A1A, 14A1B, 14A2, 14B, 15A, 15B, 15C, 16A, 16B, 17A1, 17A2, 17B, 18A1, 18A2, 18B, 18C, 19, 20A, 20B, 21A, 21B, 2A, 2B, 3A, 3B, 3C, 4A, 4B, 5A1, 5A2, 5A3, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -2359,6 +2474,11 @@
           <t>252</t>
         </is>
       </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 2A, 2B, 3, 4, 5A, 5B, 6</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -2366,6 +2486,11 @@
           <t>253</t>
         </is>
       </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>10, 11A, 11B, 11C, 12, 13, 1A, 1B, 1C, 2A, 2B, 2C, 3, 4, 5, 6, 7, 8A, 8B, 8C, 8D, 9A, 9B, 9C</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -2373,6 +2498,11 @@
           <t>254</t>
         </is>
       </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 11C, 11D, 11E, 11F, 11G, 11H, 11I, 12, 13, 14A, 14B, 15A, 15B, 15C, 16A, 16B, 2A1, 2A2, 2B, 3, 4, 5A, 5B, 6A, 6B, 7A, 7B, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -2380,6 +2510,11 @@
           <t>255</t>
         </is>
       </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13A, 13B1A1, 13B1A2, 13B1A3, 13B1B, 13B2, 13C, 13D1, 13D2, 14, 15A1A, 15A1B, 15A2A, 15A2B, 15B, 16, 17A, 17B1, 17B2A, 17B2B, 18, 19, 2, 20, 21, 22, 23A, 23B, 23C, 24, 3, 4, 5A, 5B1, 5B2, 5C, 5D1A, 5D1B, 5D2, 6, 7A1, 7A2A, 7A2B, 7B, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -2387,6 +2522,11 @@
           <t>256</t>
         </is>
       </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -2394,6 +2534,11 @@
           <t>257</t>
         </is>
       </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11, 12, 2A, 2B, 2C, 2D, 2E, 2F, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -2401,6 +2546,11 @@
           <t>258</t>
         </is>
       </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -2408,6 +2558,11 @@
           <t>259</t>
         </is>
       </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 3, 4A, 4B, 4C, 5, 6, 7A, 7B</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -2415,6 +2570,11 @@
           <t>26</t>
         </is>
       </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -2422,6 +2582,11 @@
           <t>260</t>
         </is>
       </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 23A, 23B, 24, 25, 26, 27, 28, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -2429,6 +2594,11 @@
           <t>261</t>
         </is>
       </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 1A, 1B, 1C, 1D, 1E, 2, 3, 4, 5, 6A, 6B, 6C, 6D, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -2436,6 +2606,11 @@
           <t>262</t>
         </is>
       </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>10, 11A, 11B, 11C, 11D, 12, 1A, 1B, 1C, 1D, 2A, 2B, 3, 4, 5, 6, 7, 8A, 8B, 9A, 9B, 9C</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -2443,6 +2618,11 @@
           <t>263</t>
         </is>
       </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 2, 3, 4, 5, 6, 7A1, 7A2, 7B, 8A, 8B, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -2450,6 +2630,11 @@
           <t>264</t>
         </is>
       </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>10, 11, 1A, 1B, 2A, 2B, 2C1, 2C2, 3A, 3B, 4A, 4B, 5A, 5B, 5C, 5D, 5E, 5F, 5G, 6, 7A, 7B, 7C, 7D, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -2457,6 +2642,11 @@
           <t>265</t>
         </is>
       </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17, 18A, 18B, 19A, 19B, 1A, 1B, 20, 21A, 21B, 22, 23A, 23B, 24, 25, 2A, 2B, 3, 4, 5, 6A, 6B, 7A, 7B, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -2464,6 +2654,11 @@
           <t>266</t>
         </is>
       </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 2A, 2B, 3A, 3B, 4, 5A, 5B, 5C, 5D, 6A, 6B, 7, 8, 9A, 9B, 9C1, 9C2, 9C3</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -2471,6 +2666,11 @@
           <t>267</t>
         </is>
       </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>10A, 10B, 10C, 10D, 11A, 11B, 11C, 12, 13, 14, 15, 16, 17, 18, 19, 1A, 1B, 1C1, 1C2, 2, 20, 21A1, 21A2, 21B, 21C, 21D, 3, 4A, 4B, 5A, 5B, 6, 7A, 7B, 8A, 8B, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -2478,6 +2678,11 @@
           <t>268</t>
         </is>
       </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13A, 13B, 14A1, 14A2, 14B, 14C, 15, 16, 17A, 17B, 18A, 18B, 19A, 19B, 2, 20, 21, 22, 23, 24, 3, 4A, 4B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -2485,6 +2690,11 @@
           <t>269</t>
         </is>
       </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A1, 12A2, 12B1, 12B2, 13, 14, 15A1, 15A2, 15B, 16, 17, 18, 19, 20, 21A1A, 21A1B1, 21B, 22, 23, 24, 25, 26, 27, 2A, 2B, 3A, 3B, 3C, 4, 5, 6, 7, 8A1, 8A2, 8B, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -2492,6 +2702,11 @@
           <t>27</t>
         </is>
       </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -2499,6 +2714,11 @@
           <t>270</t>
         </is>
       </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A, 12B, 12C, 12D, 12E, 13A, 13B, 13C, 14A, 14B, 15A, 15B, 15C, 15D, 15E, 15F, 15G, 2, 3A, 3B, 4, 5, 6A, 6B, 6C, 6D, 7, 8, 9A, 9B, 9C, 9D</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -2506,6 +2726,11 @@
           <t>271</t>
         </is>
       </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -2513,6 +2738,11 @@
           <t>272</t>
         </is>
       </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13A1, 13A2, 13A3, 13A4, 13B, 13C, 13D, 13E, 13F, 14, 15A1, 15A2, 15B, 15C, 16A, 16B, 17A, 17B, 18A, 18B, 19, 201A1, 201A2, 20A, 20B1A, 20B1B, 20B1C, 20B1D, 20B2, 20C1, 20C2, 20D, 20E, 20F, 20G1, 20G2, 20G3, 20G4, 20G5, 20G6, 20G7, 20H1, 20H2, 20H3, 20H4, 20H5, 20H6, 20IB, 20J, 20K, 20L, 21A1, 21A2, 21A3, 21A4, 21A5, 21A6, 21A7, 21B, 22, 23A, 23B1, 23B2, 2A, 2B, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -2520,6 +2750,11 @@
           <t>273</t>
         </is>
       </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13A, 13B, 13C, 13D, 13E, 14, 15, 16, 17A, 17B, 17C, 17D, 1A, 1B, 2A, 2B, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -2527,6 +2762,11 @@
           <t>274</t>
         </is>
       </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 1A, 1B, 1C, 1D, 1E, 1F, 1G, 2, 3, 4, 5, 6, 7A, 7B, 7C, 7D, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -2534,6 +2774,11 @@
           <t>275</t>
         </is>
       </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B1, 11B2, 12, 13, 14, 15A, 15B, 16, 17, 18A, 18B, 19A1, 19A2, 19A3, 19B1, 19B2, 19B3, 2, 20A, 20B1A1, 20B1A2, 20B2, 21, 3A, 3B, 3C, 4, 5, 6, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -2541,6 +2786,11 @@
           <t>276</t>
         </is>
       </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>10A, 10B1, 10B2, 10C, 11, 1A, 1B, 1C, 1D, 1E, 2, 3, 4, 5A, 5B1, 5B2, 6A, 6B, 7, 8A, 8B, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -2548,6 +2798,11 @@
           <t>277</t>
         </is>
       </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11, 2, 3, 4A, 4B, 5, 6A, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -2555,6 +2810,11 @@
           <t>278</t>
         </is>
       </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 2A, 2B, 3, 4, 5, 6, 7A, 7B, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -2562,6 +2822,11 @@
           <t>279</t>
         </is>
       </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2, 3A1, 3A2, 3A3, 3B, 3C, 4, 5, 6A1, 6A2, 6B, 7, 8A, 8B, 8C, 8D, 9</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -2569,6 +2834,11 @@
           <t>28</t>
         </is>
       </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -2576,6 +2846,11 @@
           <t>280</t>
         </is>
       </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>10A, 10B, 11A, 11B, 12, 13, 14A, 14B, 15, 16A, 16B, 16C, 17, 18A, 18B1, 18B2, 18C, 19A1, 19A2, 19A3, 19B, 1A1, 1A2, 1A3, 1B, 2, 20, 21, 3A1, 3A2, 3B1, 3B2, 3B3, 4, 5A, 5B, 6, 7A, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -2583,6 +2858,11 @@
           <t>281</t>
         </is>
       </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15A, 15B1, 15B2, 15B3, 16, 17, 2A, 2B, 3A, 3B, 3C, 4A, 4B, 4C, 5A, 5B, 6, 7A, 7B1, 7B2, 7B3, 7C, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -2590,6 +2870,11 @@
           <t>282</t>
         </is>
       </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -2597,6 +2882,11 @@
           <t>283</t>
         </is>
       </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -2604,6 +2894,11 @@
           <t>284</t>
         </is>
       </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -2611,6 +2906,11 @@
           <t>285</t>
         </is>
       </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -2618,6 +2918,11 @@
           <t>286</t>
         </is>
       </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>1, 10, 2A, 2B, 3, 4A, 4B2, 5, 6, 7, 8, 9, 9A</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -2625,6 +2930,11 @@
           <t>287</t>
         </is>
       </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>1, 100A, 100B, 100C, 10A, 10B, 11, 12, 13, 14, 15, 16, 17A, 17B, 17C, 17D, 17E, 18, 19, 2, 20, 21, 22A1, 22A2, 22B, 23A, 23B, 23C, 24, 25A, 25B, 26, 27A, 27B, 27C1, 27C2, 27C3, 27D, 27E, 28A, 28B, 29A, 29B, 3, 30, 31, 32, 33A, 33B, 33C, 34, 35, 36, 37, 38, 39, 4, 40A, 40B, 40C, 41, 42, 43, 44, 45A, 45B1, 45B2, 46, 47A, 47B, 48, 49A, 49B, 50A1, 50A2, 50B1, 50B2, 51, 52, 53, 54, 55, 56A, 56B, 57, 58, 59, 5A, 5B, 5C, 6, 60A, 60B, 61, 62A, 62B, 63, 64A, 64B, 65, 66, 67, 68, 69, 7, 70, 71, 72A1, 72A2, 72B1, 72B2, 72B3, 73, 74A, 74B, 75A1, 75A2, 75B, 76, 77A, 77B, 78, 79, 80, 81, 82, 83, 84, 85, 86, 87A, 87B, 88, 89A, 89B, 8A, 8B1, 8B2, 90, 91, 92, 93, 94, 95, 96A, 96B, 96C, 96D, 97, 98, 99, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -2632,6 +2942,11 @@
           <t>288</t>
         </is>
       </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 3C, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -2639,6 +2954,11 @@
           <t>289</t>
         </is>
       </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -2646,6 +2966,11 @@
           <t>29</t>
         </is>
       </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -2653,6 +2978,11 @@
           <t>290</t>
         </is>
       </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -2660,6 +2990,11 @@
           <t>291</t>
         </is>
       </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -2667,6 +3002,11 @@
           <t>292</t>
         </is>
       </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4, 5A, 5B, 6</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -2674,6 +3014,11 @@
           <t>293</t>
         </is>
       </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -2681,6 +3026,11 @@
           <t>294</t>
         </is>
       </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -2688,6 +3038,11 @@
           <t>295</t>
         </is>
       </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 4C, 4D, 5A, 5B, 5C, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -2695,6 +3050,11 @@
           <t>296</t>
         </is>
       </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 10C, 10D, 2, 3, 4, 5, 6, 7A, 7B, 7C, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -2702,6 +3062,11 @@
           <t>297</t>
         </is>
       </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -2709,6 +3074,11 @@
           <t>298</t>
         </is>
       </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 3C, 4, 5A, 5B</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -2716,6 +3086,11 @@
           <t>299</t>
         </is>
       </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 5</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -2723,6 +3098,11 @@
           <t>3</t>
         </is>
       </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -2730,6 +3110,11 @@
           <t>30</t>
         </is>
       </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11, 12, 13, 14, 15, 16, 17, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -2737,6 +3122,11 @@
           <t>300</t>
         </is>
       </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -2744,6 +3134,11 @@
           <t>301</t>
         </is>
       </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11, 12, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -2751,6 +3146,11 @@
           <t>302</t>
         </is>
       </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 1A, 1B, 1C, 2, 3A, 3B, 4A, 4B, 5A, 5B, 6A, 6B, 7A, 7B, 7C, 8A, 8B, 8C, 9</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -2758,6 +3158,11 @@
           <t>303</t>
         </is>
       </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -2765,6 +3170,11 @@
           <t>304</t>
         </is>
       </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -2772,6 +3182,11 @@
           <t>305</t>
         </is>
       </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -2779,6 +3194,11 @@
           <t>306</t>
         </is>
       </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -2786,6 +3206,11 @@
           <t>307</t>
         </is>
       </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A1, 2A2, 2A3, 2A4, 2B, 3A, 3B, 3C1A, 3C1B, 3C2, 4A, 4B, 5A, 5B1, 5B2, 6A1, 6A2, 6A3, 6B, 7A1, 7A2, 7B1, 7B2, 7C1, 7C2, 8A, 8B, 8C</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -2793,6 +3218,11 @@
           <t>308</t>
         </is>
       </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B1, 2B2, 3A, 3B1A, 3B2, 4A, 4B, 5A, 5B, 6A, 6B, 7</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -2800,6 +3230,11 @@
           <t>309</t>
         </is>
       </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3A1, 3A2, 3B, 4A1, 4A2, 4B1, 4B2, 5A, 5B, 5C, 5D, 6A1A, 6A1B, 6A2A, 6A2B, 6B1A, 6B1B, 6B2, 6C1, 6C2, 6C3, 6D1A1, 6D1A2, 6D2, 6E1, 6E2, 6E3, 6F, 6G, 7</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -2807,6 +3242,11 @@
           <t>31</t>
         </is>
       </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -2814,6 +3254,11 @@
           <t>310</t>
         </is>
       </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 2, 3, 4A, 4B, 5</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -2821,6 +3266,11 @@
           <t>311</t>
         </is>
       </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 2A, 2B, 2C, 2D, 2E, 2F, 2G, 2H, 2I, 3</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -2828,11 +3278,21 @@
           <t>312</t>
         </is>
       </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 2C, 3A, 3B, 3C, 3D, 3E, 3F, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
           <t>313</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1, 1B2, 2A, 2B, 3A, 3B, 3C, 4A1, 4A2, 4B, 4C, 5A1A, 5A1B, 5A2, 5B, 5C, 6A, 6B, 7, 8A, 8B, 8C, 8D, 9</t>
         </is>
       </c>
     </row>

</xml_diff>